<commit_message>
actulització base de dades partits 16 de desembre
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D47DF98E-6B63-44D3-BC1E-A7471AC86E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11422B43-3CE7-9C4F-91AE-2CB889287338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="4" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="75">
   <si>
     <t>code_h</t>
   </si>
@@ -48,9 +48,6 @@
     <t>code_a</t>
   </si>
   <si>
-    <t>date</t>
-  </si>
-  <si>
     <t>round</t>
   </si>
   <si>
@@ -91,18 +88,201 @@
   </si>
   <si>
     <t>category</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>U2025</t>
+  </si>
+  <si>
+    <t>E2025</t>
+  </si>
+  <si>
+    <t>PRS</t>
+  </si>
+  <si>
+    <t>BAR</t>
+  </si>
+  <si>
+    <t>LJU</t>
+  </si>
+  <si>
+    <t>JER</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>Barcelona</t>
+  </si>
+  <si>
+    <t>Cedevita Olimpija</t>
+  </si>
+  <si>
+    <t>Hapoel Jerusalem</t>
+  </si>
+  <si>
+    <t>Pablo Campoy</t>
+  </si>
+  <si>
+    <t>Oriol Garcia</t>
+  </si>
+  <si>
+    <t>Mario Enjuanes</t>
+  </si>
+  <si>
+    <t>Marc Ventura</t>
+  </si>
+  <si>
+    <t>Hector Guillen</t>
+  </si>
+  <si>
+    <t>Xavier Mateu</t>
+  </si>
+  <si>
+    <t>Eloi Verge</t>
+  </si>
+  <si>
+    <t>Oscar Cuesta</t>
+  </si>
+  <si>
+    <t>Nerea Fraile</t>
+  </si>
+  <si>
+    <t>DYLAN YAMDJEU SANGOUNGOU</t>
+  </si>
+  <si>
+    <t>JIMMY MOLLET</t>
+  </si>
+  <si>
+    <t>BASTIEN BONNETON</t>
+  </si>
+  <si>
+    <t>CYRIL LONGELIN</t>
+  </si>
+  <si>
+    <t>MAGALI CARTIER</t>
+  </si>
+  <si>
+    <t>AXEL QUENEY</t>
+  </si>
+  <si>
+    <t>BRIAN PETER</t>
+  </si>
+  <si>
+    <t>DJAMEL SOUDANI</t>
+  </si>
+  <si>
+    <t>CHRISTIAN MOLLET</t>
+  </si>
+  <si>
+    <t>SANDRA PRINCELLE</t>
+  </si>
+  <si>
+    <t>PATRICK JOLIVET</t>
+  </si>
+  <si>
+    <t>PIERRE BERNARDO</t>
+  </si>
+  <si>
+    <t>JESUS LOPEZ</t>
+  </si>
+  <si>
+    <t>POL FRANQUESA</t>
+  </si>
+  <si>
+    <t>ROBERTO BAÑOS</t>
+  </si>
+  <si>
+    <t>MARC BAYO</t>
+  </si>
+  <si>
+    <t>LLUIS ESPINOSA</t>
+  </si>
+  <si>
+    <t>RICARD MONGE</t>
+  </si>
+  <si>
+    <t>MARIA JOSE SERRANO</t>
+  </si>
+  <si>
+    <t>CARLOS MARTIN</t>
+  </si>
+  <si>
+    <t>MANEL LUENGO</t>
+  </si>
+  <si>
+    <t>FRANCIS RUIZ</t>
+  </si>
+  <si>
+    <t>ADRIA RUBIROLA</t>
+  </si>
+  <si>
+    <t>LAILA GONELL</t>
+  </si>
+  <si>
+    <t>NEŽA JUG</t>
+  </si>
+  <si>
+    <t>ZIGA JANEZ</t>
+  </si>
+  <si>
+    <t>ALENKA MARKIC</t>
+  </si>
+  <si>
+    <t>SILVO MARKIC</t>
+  </si>
+  <si>
+    <t>KARMEN BELSAK</t>
+  </si>
+  <si>
+    <t>MATJAZ PODLESNIK</t>
+  </si>
+  <si>
+    <t>GORAN HODZIC</t>
+  </si>
+  <si>
+    <t>ANA JUG</t>
+  </si>
+  <si>
+    <t>MATIC MARKIC</t>
+  </si>
+  <si>
+    <t>ANDREJ STRUKELJ</t>
+  </si>
+  <si>
+    <t>URBAN VERBIC</t>
+  </si>
+  <si>
+    <t>GASPER KOLMAN</t>
+  </si>
+  <si>
+    <t>ZIGA BENKO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -114,7 +294,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -122,17 +302,240 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="11">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -146,36 +549,41 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:G2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:G2" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1404C5E0-6886-4CE4-90B6-B0B18B1A65AF}" name="game_code"/>
-    <tableColumn id="2" xr3:uid="{F7E24D2C-A0CE-449B-BC4C-C95243A6E984}" name="code_h"/>
-    <tableColumn id="3" xr3:uid="{6E5975D4-6595-4C17-AB73-8744367F6A19}" name="code_a"/>
-    <tableColumn id="4" xr3:uid="{96895ED8-5783-4AE4-AD21-622BA87C414A}" name="date"/>
-    <tableColumn id="5" xr3:uid="{C142F6C7-57D8-4529-8A58-0A322148FE5E}" name="round"/>
-    <tableColumn id="6" xr3:uid="{E6DB1CD4-0191-459F-9331-BEF47D42C436}" name="competition_code"/>
-    <tableColumn id="7" xr3:uid="{60F9E97B-C247-488D-B753-F79D1BDD7D79}" name="num_actions"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:I3" totalsRowShown="0">
+  <autoFilter ref="A1:I3" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I3">
+    <sortCondition ref="F1:F3"/>
+  </sortState>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{1404C5E0-6886-4CE4-90B6-B0B18B1A65AF}" name="game_code" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{F7E24D2C-A0CE-449B-BC4C-C95243A6E984}" name="code_h" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{6E5975D4-6595-4C17-AB73-8744367F6A19}" name="code_a" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{CFA8E310-068A-7140-9213-5657FEBFAB3A}" name="year" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{AC18B8EC-8A7C-2245-AA3B-DF6BEFE4F9D6}" name="month" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{96895ED8-5783-4AE4-AD21-622BA87C414A}" name="day" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{C142F6C7-57D8-4529-8A58-0A322148FE5E}" name="round" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{E6DB1CD4-0191-459F-9331-BEF47D42C436}" name="competition_code" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{60F9E97B-C247-488D-B753-F79D1BDD7D79}" name="num_actions" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:C2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:C2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:C5" totalsRowShown="0">
+  <autoFilter ref="A1:C5" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="2" xr3:uid="{138ECFBF-CE75-490C-BC44-2803CEC43525}" name="pbp_name"/>
-    <tableColumn id="3" xr3:uid="{6638DC74-71D4-4412-937F-A2EFB7ED9C16}" name="discord_channel_id"/>
+    <tableColumn id="3" xr3:uid="{6638DC74-71D4-4412-937F-A2EFB7ED9C16}" name="discord_channel_id" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{14980971-F19F-4658-A94B-998FE494D814}" name="Table3" displayName="Table3" ref="A1:B2" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="A1:B2" xr:uid="{14980971-F19F-4658-A94B-998FE494D814}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{14980971-F19F-4658-A94B-998FE494D814}" name="Table3" displayName="Table3" ref="A1:B53" totalsRowShown="0">
+  <autoFilter ref="A1:B53" xr:uid="{14980971-F19F-4658-A94B-998FE494D814}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E928ABD3-4C33-4D2A-A2E5-B849CBD6D2FD}" name="team_code"/>
     <tableColumn id="2" xr3:uid="{85523702-4932-4E93-9E20-C5013B1376EF}" name="name"/>
@@ -185,11 +593,11 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A94C063E-C8B8-4C57-8C73-8225A8C83E6D}" name="Table4" displayName="Table4" ref="A1:B2" totalsRowShown="0">
-  <autoFilter ref="A1:B2" xr:uid="{A94C063E-C8B8-4C57-8C73-8225A8C83E6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A94C063E-C8B8-4C57-8C73-8225A8C83E6D}" name="Table4" displayName="Table4" ref="A1:B10" totalsRowShown="0">
+  <autoFilter ref="A1:B10" xr:uid="{A94C063E-C8B8-4C57-8C73-8225A8C83E6D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{2F07979F-4A38-4C38-B72B-159C21B04AE0}" name="name"/>
-    <tableColumn id="2" xr3:uid="{48C33198-8C8F-40A5-B369-CD15AEA96EC8}" name="discord_id"/>
+    <tableColumn id="2" xr3:uid="{48C33198-8C8F-40A5-B369-CD15AEA96EC8}" name="discord_id" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -528,19 +936,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.453125" customWidth="1"/>
-    <col min="2" max="2" width="10.26953125" customWidth="1"/>
-    <col min="3" max="3" width="10.36328125" customWidth="1"/>
-    <col min="6" max="6" width="20.1796875" customWidth="1"/>
-    <col min="7" max="7" width="14.90625" customWidth="1"/>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="2" max="5" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.1640625" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -549,17 +956,77 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>102</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E2" s="1">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1">
+        <v>16</v>
+      </c>
+      <c r="G2" s="1">
         <v>11</v>
       </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
+      <c r="H2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>156</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2025</v>
+      </c>
+      <c r="E3" s="1">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1">
+        <v>16</v>
+      </c>
+      <c r="G3" s="1">
+        <v>16</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -571,23 +1038,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
-    <col min="2" max="2" width="13.36328125" customWidth="1"/>
-    <col min="3" max="3" width="22.26953125" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
-        <v>8</v>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2">
+        <v>8.8514831092981299E+17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2">
+        <v>8.8493377688974899E+17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="2">
+        <v>8.8514917923884198E+17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1.28780243194557E+18</v>
       </c>
     </row>
   </sheetData>
@@ -600,19 +1112,390 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B53"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>23</v>
+      </c>
+      <c r="B37" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -625,19 +1508,91 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.6328125" customWidth="1"/>
-    <col min="2" max="2" width="14.36328125" customWidth="1"/>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
-        <v>10</v>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="3">
+        <v>8.8550585082171802E+17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="3">
+        <v>8.9314831284320998E+17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="3">
+        <v>8.9314196703322906E+17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="3">
+        <v>8.5194742619255603E+17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="3">
+        <v>9.0003431883396698E+17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1.20477629114063E+18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1.34430823875294E+18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="3">
+        <v>6.9749520416872806E+17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1.42765367961951E+18</v>
       </c>
     </row>
   </sheetData>
@@ -651,34 +1606,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.6328125" customWidth="1"/>
-    <col min="2" max="2" width="19.81640625" customWidth="1"/>
-    <col min="3" max="7" width="10.6328125" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" customWidth="1"/>
+    <col min="3" max="7" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>15</v>
-      </c>
-      <c r="G1" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
afegir uscs jerusalem a base de dades
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11422B43-3CE7-9C4F-91AE-2CB889287338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59854FC1-E863-403D-94EF-90F1A90364DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="4" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="90">
   <si>
     <t>code_h</t>
   </si>
@@ -265,13 +265,58 @@
   </si>
   <si>
     <t>ZIGA BENKO</t>
+  </si>
+  <si>
+    <t>MILOS MOSIC</t>
+  </si>
+  <si>
+    <t>IVAN MOSIC</t>
+  </si>
+  <si>
+    <t>MIODRAG STOJANOVIC</t>
+  </si>
+  <si>
+    <t>PETAR VASILJEVIC</t>
+  </si>
+  <si>
+    <t>PREDRAG VASILJEVIC</t>
+  </si>
+  <si>
+    <t>IVANA VASILJEVIC</t>
+  </si>
+  <si>
+    <t>MILICA STOSIC</t>
+  </si>
+  <si>
+    <t>JOVANA VESKOVIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANA KRSTIC </t>
+  </si>
+  <si>
+    <t>MILAN KVRGIC</t>
+  </si>
+  <si>
+    <t>LUKA ANDRIC</t>
+  </si>
+  <si>
+    <t>MARKO BOZIC</t>
+  </si>
+  <si>
+    <t>SARA PROJOVIC</t>
+  </si>
+  <si>
+    <t>MARIJA SAVIC</t>
+  </si>
+  <si>
+    <t>SARA MILICIC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -283,6 +328,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -321,11 +372,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -937,15 +991,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
-    <col min="2" max="5" width="10.33203125" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="5" width="10.36328125" customWidth="1"/>
+    <col min="8" max="8" width="20.1796875" customWidth="1"/>
+    <col min="9" max="9" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -974,7 +1028,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>102</v>
       </c>
@@ -1001,7 +1055,7 @@
       </c>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>156</v>
       </c>
@@ -1039,15 +1093,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" customWidth="1"/>
-    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+    <col min="3" max="3" width="22.36328125" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1058,7 +1112,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1069,7 +1123,7 @@
         <v>8.8514831092981299E+17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1080,7 +1134,7 @@
         <v>8.8493377688974899E+17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -1091,7 +1145,7 @@
         <v>8.8514917923884198E+17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1113,13 +1167,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
   <dimension ref="A1:B53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1127,7 +1181,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1135,7 +1189,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1143,7 +1197,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1151,7 +1205,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1159,7 +1213,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1167,7 +1221,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1175,7 +1229,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1183,7 +1237,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1191,7 +1245,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1199,7 +1253,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1207,7 +1261,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1215,7 +1269,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1223,7 +1277,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1231,7 +1285,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1239,7 +1293,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1247,7 +1301,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1255,7 +1309,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1263,7 +1317,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1271,7 +1325,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1279,7 +1333,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -1287,7 +1341,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1295,7 +1349,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -1303,7 +1357,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1311,7 +1365,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -1319,7 +1373,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1327,7 +1381,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -1335,7 +1389,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -1343,7 +1397,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1351,7 +1405,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1359,7 +1413,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -1367,7 +1421,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -1375,7 +1429,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -1383,7 +1437,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -1391,7 +1445,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -1399,7 +1453,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -1407,7 +1461,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -1415,7 +1469,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>23</v>
       </c>
@@ -1423,79 +1477,124 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B39" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B40" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B41" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B42" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B43" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B44" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B45" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B46" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B47" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B48" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B49" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B50" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B51" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B52" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>24</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1509,13 +1608,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1523,7 +1622,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1531,7 +1630,7 @@
         <v>8.8550585082171802E+17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1539,7 +1638,7 @@
         <v>8.9314831284320998E+17</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -1547,7 +1646,7 @@
         <v>8.9314196703322906E+17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1555,7 +1654,7 @@
         <v>8.5194742619255603E+17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -1563,7 +1662,7 @@
         <v>9.0003431883396698E+17</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -1571,7 +1670,7 @@
         <v>1.20477629114063E+18</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -1579,7 +1678,7 @@
         <v>1.34430823875294E+18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -1587,7 +1686,7 @@
         <v>6.9749520416872806E+17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1606,14 +1705,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" customWidth="1"/>
-    <col min="3" max="7" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.6328125" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" customWidth="1"/>
+    <col min="3" max="7" width="10.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
modificacio valors enters molt llargs base de dades i primers passos per automitzar bé
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59854FC1-E863-403D-94EF-90F1A90364DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7BA6DF9-2D33-0A4B-BE0C-B6392E13E953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="4" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="103">
   <si>
     <t>code_h</t>
   </si>
@@ -310,24 +310,57 @@
   </si>
   <si>
     <t>SARA MILICIC</t>
+  </si>
+  <si>
+    <t>885148310929813517</t>
+  </si>
+  <si>
+    <t>884933776889749504</t>
+  </si>
+  <si>
+    <t>885149179238842448</t>
+  </si>
+  <si>
+    <t>1287802431945576448</t>
+  </si>
+  <si>
+    <t>885505850821718037</t>
+  </si>
+  <si>
+    <t>893148312843210833</t>
+  </si>
+  <si>
+    <t>893141967033229344</t>
+  </si>
+  <si>
+    <t>851947426192556062</t>
+  </si>
+  <si>
+    <t>900034318833967154</t>
+  </si>
+  <si>
+    <t>1204776291140636764</t>
+  </si>
+  <si>
+    <t>1344308238752944208</t>
+  </si>
+  <si>
+    <t>697495204168728586</t>
+  </si>
+  <si>
+    <t>1427653679619510383</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -372,14 +405,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,7 +423,7 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -991,15 +1025,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.453125" customWidth="1"/>
-    <col min="2" max="5" width="10.36328125" customWidth="1"/>
-    <col min="8" max="8" width="20.1796875" customWidth="1"/>
-    <col min="9" max="9" width="14.81640625" customWidth="1"/>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="2" max="5" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="20.1640625" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1028,7 +1062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>102</v>
       </c>
@@ -1055,7 +1089,7 @@
       </c>
       <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>156</v>
       </c>
@@ -1093,15 +1127,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" customWidth="1"/>
-    <col min="2" max="2" width="16.81640625" customWidth="1"/>
-    <col min="3" max="3" width="22.36328125" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1112,48 +1147,48 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="2">
-        <v>8.8514831092981299E+17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C2" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>22</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="2">
-        <v>8.8493377688974899E+17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C3" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="2">
-        <v>8.8514917923884198E+17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C4" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="2">
-        <v>1.28780243194557E+18</v>
+      <c r="C5" s="4" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1167,13 +1202,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
   <dimension ref="A1:B53"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6328125" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1181,7 +1216,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1189,7 +1224,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1197,7 +1232,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1205,7 +1240,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1213,7 +1248,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1221,7 +1256,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1229,7 +1264,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1237,7 +1272,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1245,7 +1280,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1253,7 +1288,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1261,7 +1296,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1269,7 +1304,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1277,7 +1312,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -1285,7 +1320,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1293,7 +1328,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1301,7 +1336,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1309,7 +1344,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1317,7 +1352,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1325,7 +1360,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1333,7 +1368,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -1341,7 +1376,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1349,7 +1384,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -1357,7 +1392,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1365,7 +1400,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -1373,7 +1408,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1381,7 +1416,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -1389,7 +1424,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>23</v>
       </c>
@@ -1397,7 +1432,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1405,7 +1440,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1413,7 +1448,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -1421,7 +1456,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -1429,7 +1464,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -1437,7 +1472,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -1445,7 +1480,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -1453,7 +1488,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -1461,7 +1496,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -1469,7 +1504,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>23</v>
       </c>
@@ -1477,123 +1512,123 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>24</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="B40" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>24</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>24</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B43" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B44" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>24</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>24</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>24</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>24</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B48" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>24</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B49" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>24</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>24</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>24</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="2" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1608,13 +1643,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
-    <col min="2" max="2" width="26.36328125" customWidth="1"/>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1622,76 +1657,76 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="3">
-        <v>8.8550585082171802E+17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B2" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="3">
-        <v>8.9314831284320998E+17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B3" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="3">
-        <v>8.9314196703322906E+17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="3">
-        <v>8.5194742619255603E+17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B5" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="3">
-        <v>9.0003431883396698E+17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B6" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="3">
-        <v>1.20477629114063E+18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B7" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="3">
-        <v>1.34430823875294E+18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B8" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="3">
-        <v>6.9749520416872806E+17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B9" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="3">
-        <v>1.42765367961951E+18</v>
+      <c r="B10" s="5" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1705,14 +1740,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.6328125" customWidth="1"/>
-    <col min="2" max="2" width="19.81640625" customWidth="1"/>
-    <col min="3" max="7" width="10.6328125" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" customWidth="1"/>
+    <col min="3" max="7" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
modificació taula Game base de dades
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7BA6DF9-2D33-0A4B-BE0C-B6392E13E953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D0A0E00-1AE6-4D4D-B9E2-464FACE47A28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="4" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="103">
   <si>
     <t>code_h</t>
   </si>
@@ -99,12 +99,6 @@
     <t>year</t>
   </si>
   <si>
-    <t>U2025</t>
-  </si>
-  <si>
-    <t>E2025</t>
-  </si>
-  <si>
     <t>PRS</t>
   </si>
   <si>
@@ -349,6 +343,12 @@
   </si>
   <si>
     <t>1427653679619510383</t>
+  </si>
+  <si>
+    <t>U2025_102</t>
+  </si>
+  <si>
+    <t>E2025_156</t>
   </si>
 </sst>
 </file>
@@ -405,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -413,61 +413,41 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -637,21 +617,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:I3" totalsRowShown="0">
-  <autoFilter ref="A1:I3" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:H3" totalsRowShown="0">
+  <autoFilter ref="A1:H3" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H3">
     <sortCondition ref="F1:F3"/>
   </sortState>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1404C5E0-6886-4CE4-90B6-B0B18B1A65AF}" name="game_code" dataDxfId="10"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{1404C5E0-6886-4CE4-90B6-B0B18B1A65AF}" name="game_code" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{F7E24D2C-A0CE-449B-BC4C-C95243A6E984}" name="code_h" dataDxfId="9"/>
     <tableColumn id="3" xr3:uid="{6E5975D4-6595-4C17-AB73-8744367F6A19}" name="code_a" dataDxfId="8"/>
     <tableColumn id="9" xr3:uid="{CFA8E310-068A-7140-9213-5657FEBFAB3A}" name="year" dataDxfId="7"/>
     <tableColumn id="8" xr3:uid="{AC18B8EC-8A7C-2245-AA3B-DF6BEFE4F9D6}" name="month" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{96895ED8-5783-4AE4-AD21-622BA87C414A}" name="day" dataDxfId="5"/>
     <tableColumn id="5" xr3:uid="{C142F6C7-57D8-4529-8A58-0A322148FE5E}" name="round" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{E6DB1CD4-0191-459F-9331-BEF47D42C436}" name="competition_code" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{60F9E97B-C247-488D-B753-F79D1BDD7D79}" name="num_actions" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{60F9E97B-C247-488D-B753-F79D1BDD7D79}" name="num_actions" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -663,7 +642,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="2" xr3:uid="{138ECFBF-CE75-490C-BC44-2803CEC43525}" name="pbp_name"/>
-    <tableColumn id="3" xr3:uid="{6638DC74-71D4-4412-937F-A2EFB7ED9C16}" name="discord_channel_id" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{6638DC74-71D4-4412-937F-A2EFB7ED9C16}" name="discord_channel_id" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -685,7 +664,7 @@
   <autoFilter ref="A1:B10" xr:uid="{A94C063E-C8B8-4C57-8C73-8225A8C83E6D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{2F07979F-4A38-4C38-B72B-159C21B04AE0}" name="name"/>
-    <tableColumn id="2" xr3:uid="{48C33198-8C8F-40A5-B369-CD15AEA96EC8}" name="discord_id" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{48C33198-8C8F-40A5-B369-CD15AEA96EC8}" name="discord_id" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1024,16 +1003,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
-    <col min="2" max="5" width="10.33203125" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="5" width="10.36328125" customWidth="1"/>
+    <col min="8" max="8" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1056,21 +1034,18 @@
         <v>2</v>
       </c>
       <c r="H1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>102</v>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D2" s="1">
         <v>2025</v>
@@ -1084,20 +1059,17 @@
       <c r="G2" s="1">
         <v>11</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>156</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1">
         <v>2025</v>
@@ -1111,10 +1083,7 @@
       <c r="G3" s="1">
         <v>16</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="1"/>
+      <c r="H3" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1127,16 +1096,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" customWidth="1"/>
-    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.1640625" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+    <col min="3" max="3" width="22.36328125" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1147,48 +1116,48 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1202,13 +1171,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
   <dimension ref="A1:B53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1216,420 +1185,420 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="B29" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>21</v>
       </c>
-      <c r="B7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="B31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>21</v>
       </c>
-      <c r="B8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B32" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>21</v>
       </c>
-      <c r="B9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>21</v>
       </c>
-      <c r="B10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="B34" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>21</v>
       </c>
-      <c r="B11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="B35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>21</v>
       </c>
-      <c r="B12" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="B36" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>21</v>
       </c>
-      <c r="B13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="B37" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>22</v>
       </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="B39" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>22</v>
       </c>
-      <c r="B15" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="B40" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>22</v>
       </c>
-      <c r="B16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B41" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>22</v>
       </c>
-      <c r="B17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="B42" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>22</v>
       </c>
-      <c r="B18" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B43" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>22</v>
       </c>
-      <c r="B19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="B44" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>22</v>
       </c>
-      <c r="B20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B45" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>22</v>
       </c>
-      <c r="B21" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B46" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>22</v>
       </c>
-      <c r="B22" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="B47" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="B48" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>22</v>
       </c>
-      <c r="B24" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="B49" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>22</v>
       </c>
-      <c r="B25" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>23</v>
-      </c>
-      <c r="B30" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>23</v>
-      </c>
-      <c r="B31" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>23</v>
-      </c>
-      <c r="B32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>23</v>
-      </c>
-      <c r="B35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>23</v>
-      </c>
-      <c r="B36" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>23</v>
-      </c>
-      <c r="B37" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>23</v>
-      </c>
-      <c r="B38" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>24</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>24</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>24</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>24</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>24</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>24</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>24</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>24</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>24</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>24</v>
-      </c>
-      <c r="B48" s="2" t="s">
+      <c r="B50" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>24</v>
-      </c>
-      <c r="B49" s="2" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>24</v>
-      </c>
-      <c r="B50" s="2" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>24</v>
-      </c>
-      <c r="B51" s="2" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>24</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="16" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>24</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1643,13 +1612,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1657,76 +1626,76 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B6" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B10" s="5" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1740,14 +1709,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.83203125" customWidth="1"/>
-    <col min="3" max="7" width="10.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.6328125" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" customWidth="1"/>
+    <col min="3" max="7" width="10.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
afegint uscs a la taula Game
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8DEB79A-14B9-6C49-A9E5-FF972E835557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739997B9-E150-42F9-AF13-DE08FFC2C450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="-1460" windowWidth="38400" windowHeight="21100" activeTab="5" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="269">
   <si>
     <t>code_h</t>
   </si>
@@ -601,9 +601,6 @@
     <t>Fenerbahce</t>
   </si>
   <si>
-    <t>884934005005373460</t>
-  </si>
-  <si>
     <t>Technical Foul</t>
   </si>
   <si>
@@ -775,9 +772,6 @@
     <t>Aris</t>
   </si>
   <si>
-    <t>E2025_211</t>
-  </si>
-  <si>
     <t>IST</t>
   </si>
   <si>
@@ -800,13 +794,67 @@
   </si>
   <si>
     <t>884933038469939200</t>
+  </si>
+  <si>
+    <t>E2025_217</t>
+  </si>
+  <si>
+    <t>PAM</t>
+  </si>
+  <si>
+    <t>Valencia Basket</t>
+  </si>
+  <si>
+    <t>Valencia</t>
+  </si>
+  <si>
+    <t>885903840971489330</t>
+  </si>
+  <si>
+    <t>data_entry</t>
+  </si>
+  <si>
+    <t>caller_1</t>
+  </si>
+  <si>
+    <t>caller_2</t>
+  </si>
+  <si>
+    <t>timer</t>
+  </si>
+  <si>
+    <t>shot_clock_operator</t>
+  </si>
+  <si>
+    <t>irs_operator</t>
+  </si>
+  <si>
+    <t>ENDER OZBEK</t>
+  </si>
+  <si>
+    <t>SERTAC DOSTEL</t>
+  </si>
+  <si>
+    <t>CAN KUTLUATA</t>
+  </si>
+  <si>
+    <t>GIZEM UNSAL</t>
+  </si>
+  <si>
+    <t>AHMET ERKASAP</t>
+  </si>
+  <si>
+    <t>MURAT KUS</t>
+  </si>
+  <si>
+    <t>1438645665340198915</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -820,6 +868,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -829,7 +883,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -865,11 +919,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -880,16 +945,149 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="15">
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
@@ -1060,27 +1258,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:G2" totalsRowShown="0">
-  <autoFilter ref="A1:G2" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:M2" totalsRowShown="0">
+  <autoFilter ref="A1:M2" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G2">
     <sortCondition ref="F1:F2"/>
   </sortState>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1404C5E0-6886-4CE4-90B6-B0B18B1A65AF}" name="game_code" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{F7E24D2C-A0CE-449B-BC4C-C95243A6E984}" name="code_h" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{6E5975D4-6595-4C17-AB73-8744367F6A19}" name="code_a" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{CFA8E310-068A-7140-9213-5657FEBFAB3A}" name="year" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{AC18B8EC-8A7C-2245-AA3B-DF6BEFE4F9D6}" name="month" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{96895ED8-5783-4AE4-AD21-622BA87C414A}" name="day" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{C142F6C7-57D8-4529-8A58-0A322148FE5E}" name="round" dataDxfId="2"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{1404C5E0-6886-4CE4-90B6-B0B18B1A65AF}" name="game_code" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{F7E24D2C-A0CE-449B-BC4C-C95243A6E984}" name="code_h" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{6E5975D4-6595-4C17-AB73-8744367F6A19}" name="code_a" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{CFA8E310-068A-7140-9213-5657FEBFAB3A}" name="year" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{AC18B8EC-8A7C-2245-AA3B-DF6BEFE4F9D6}" name="month" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{96895ED8-5783-4AE4-AD21-622BA87C414A}" name="day" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{C142F6C7-57D8-4529-8A58-0A322148FE5E}" name="round" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{ADE7E51A-081F-4C48-B084-2B62E97062EA}" name="data_entry" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{158B2440-9D42-49A2-B9A5-DE39CB23F724}" name="caller_1" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{1D3F1CA7-134A-4A3C-9FA3-63DB5F051E22}" name="caller_2" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{4D83FFAB-5962-44CB-9AA8-FEF22DF1489B}" name="timer" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{00145A72-6E33-46B2-8BE6-AD8BB8B9CE0C}" name="shot_clock_operator" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{A35F176E-A5B4-4367-92E3-04B2F6CBD3A6}" name="irs_operator" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D23" totalsRowShown="0">
-  <autoFilter ref="A1:D23" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D24" totalsRowShown="0">
+  <autoFilter ref="A1:D24" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="4" xr3:uid="{760465A9-3097-934B-AB04-6544582DE0F4}" name="team_name"/>
@@ -1463,15 +1667,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
-    <col min="2" max="5" width="10.33203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.26953125" customWidth="1"/>
+    <col min="13" max="13" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -1493,16 +1707,34 @@
       <c r="G1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" t="s">
+        <v>256</v>
+      </c>
+      <c r="I1" t="s">
+        <v>257</v>
+      </c>
+      <c r="J1" t="s">
+        <v>258</v>
+      </c>
+      <c r="K1" t="s">
+        <v>259</v>
+      </c>
+      <c r="L1" t="s">
+        <v>260</v>
+      </c>
+      <c r="M1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>245</v>
+        <v>184</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="D2" s="1">
         <v>2026</v>
@@ -1511,13 +1743,32 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="1">
         <v>22</v>
       </c>
+      <c r="H2" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>267</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1527,23 +1778,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.1640625" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
@@ -1552,12 +1803,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -1566,12 +1817,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
@@ -1580,12 +1831,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -1594,12 +1845,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -1608,12 +1859,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>141</v>
       </c>
       <c r="B6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C6" t="s">
         <v>143</v>
@@ -1622,12 +1873,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>142</v>
       </c>
       <c r="B7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C7" t="s">
         <v>144</v>
@@ -1636,12 +1887,12 @@
         <v>146</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C8" t="s">
         <v>150</v>
@@ -1650,12 +1901,12 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>148</v>
       </c>
       <c r="B9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C9" t="s">
         <v>149</v>
@@ -1664,12 +1915,12 @@
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>160</v>
       </c>
       <c r="B10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C10" t="s">
         <v>164</v>
@@ -1678,12 +1929,12 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>161</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C11" t="s">
         <v>165</v>
@@ -1692,12 +1943,12 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>162</v>
       </c>
       <c r="B12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C12" t="s">
         <v>166</v>
@@ -1706,12 +1957,12 @@
         <v>170</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>163</v>
       </c>
       <c r="B13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C13" t="s">
         <v>167</v>
@@ -1720,12 +1971,12 @@
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>172</v>
       </c>
       <c r="B14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C14" t="s">
         <v>176</v>
@@ -1734,12 +1985,12 @@
         <v>180</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>173</v>
       </c>
       <c r="B15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C15" t="s">
         <v>177</v>
@@ -1748,12 +1999,12 @@
         <v>181</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>174</v>
       </c>
       <c r="B16" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C16" t="s">
         <v>178</v>
@@ -1762,12 +2013,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>175</v>
       </c>
       <c r="B17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C17" t="s">
         <v>179</v>
@@ -1776,88 +2027,102 @@
         <v>183</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>184</v>
       </c>
       <c r="B18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C18" t="s">
         <v>185</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>187</v>
+      </c>
+      <c r="B19" t="s">
+        <v>224</v>
+      </c>
+      <c r="C19" t="s">
         <v>188</v>
       </c>
-      <c r="B19" t="s">
-        <v>225</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>235</v>
+      </c>
+      <c r="B20" t="s">
         <v>236</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>237</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="D20" s="4" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>240</v>
+      </c>
+      <c r="B21" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="C21" t="s">
+        <v>242</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="B21" t="s">
-        <v>240</v>
-      </c>
-      <c r="C21" t="s">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>243</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
         <v>245</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>247</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>244</v>
+      </c>
+      <c r="B23" t="s">
         <v>246</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>248</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D23" s="4" t="s">
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>252</v>
+      </c>
+      <c r="B24" t="s">
+        <v>253</v>
+      </c>
+      <c r="C24" t="s">
+        <v>254</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -1871,13 +2136,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
   <dimension ref="A1:B63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1885,7 +2150,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1893,7 +2158,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1901,7 +2166,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1909,7 +2174,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1917,7 +2182,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1925,7 +2190,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1933,7 +2198,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1941,7 +2206,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1949,7 +2214,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1957,7 +2222,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1965,7 +2230,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1973,7 +2238,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1981,7 +2246,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1989,7 +2254,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1997,7 +2262,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -2005,7 +2270,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -2013,7 +2278,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2021,7 +2286,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -2029,7 +2294,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -2037,7 +2302,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -2045,7 +2310,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -2053,7 +2318,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -2061,7 +2326,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -2069,7 +2334,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -2077,7 +2342,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -2085,7 +2350,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -2093,7 +2358,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -2101,7 +2366,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -2109,7 +2374,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -2117,7 +2382,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -2125,7 +2390,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>18</v>
       </c>
@@ -2133,7 +2398,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -2141,7 +2406,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -2149,7 +2414,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>18</v>
       </c>
@@ -2157,7 +2422,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>18</v>
       </c>
@@ -2165,7 +2430,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>18</v>
       </c>
@@ -2173,7 +2438,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>18</v>
       </c>
@@ -2181,7 +2446,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -2189,7 +2454,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>19</v>
       </c>
@@ -2197,7 +2462,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>19</v>
       </c>
@@ -2205,7 +2470,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>19</v>
       </c>
@@ -2213,7 +2478,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>19</v>
       </c>
@@ -2221,7 +2486,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -2229,7 +2494,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>19</v>
       </c>
@@ -2237,7 +2502,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -2245,7 +2510,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -2253,7 +2518,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>19</v>
       </c>
@@ -2261,7 +2526,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>19</v>
       </c>
@@ -2269,7 +2534,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>19</v>
       </c>
@@ -2277,7 +2542,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>19</v>
       </c>
@@ -2285,7 +2550,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -2293,7 +2558,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>19</v>
       </c>
@@ -2301,84 +2566,84 @@
         <v>75</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>172</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>172</v>
       </c>
       <c r="B55" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>172</v>
       </c>
       <c r="B56" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>172</v>
       </c>
       <c r="B57" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>172</v>
       </c>
       <c r="B58" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>172</v>
       </c>
       <c r="B59" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>172</v>
       </c>
       <c r="B60" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>172</v>
       </c>
       <c r="B61" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>172</v>
       </c>
       <c r="B62" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>172</v>
       </c>
       <c r="B63" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2392,13 +2657,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -2406,73 +2671,73 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>88</v>
@@ -2489,41 +2754,41 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C1" t="s">
         <v>9</v>
       </c>
       <c r="D1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" t="s">
         <v>194</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>195</v>
-      </c>
-      <c r="F1" t="s">
-        <v>196</v>
       </c>
       <c r="G1" t="s">
         <v>10</v>
@@ -2532,7 +2797,7 @@
         <v>11</v>
       </c>
       <c r="I1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J1" t="s">
         <v>12</v>
@@ -2541,10 +2806,10 @@
         <v>89</v>
       </c>
       <c r="L1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="M1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -2558,13 +2823,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E819B3A5-8F6D-6649-8C82-B76A24B61AC2}">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>90</v>
       </c>
@@ -2572,7 +2837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -2580,7 +2845,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>92</v>
       </c>
@@ -2588,7 +2853,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -2596,7 +2861,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -2604,7 +2869,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -2612,7 +2877,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -2620,7 +2885,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>154</v>
       </c>
@@ -2628,7 +2893,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -2636,7 +2901,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>98</v>
       </c>
@@ -2644,7 +2909,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>99</v>
       </c>
@@ -2652,7 +2917,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>100</v>
       </c>
@@ -2660,7 +2925,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>101</v>
       </c>
@@ -2668,7 +2933,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>102</v>
       </c>
@@ -2676,7 +2941,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>103</v>
       </c>
@@ -2684,7 +2949,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>104</v>
       </c>
@@ -2692,7 +2957,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>155</v>
       </c>
@@ -2700,7 +2965,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>105</v>
       </c>
@@ -2708,7 +2973,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -2716,7 +2981,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>107</v>
       </c>
@@ -2724,7 +2989,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2732,7 +2997,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>126</v>
       </c>
@@ -2740,7 +3005,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>156</v>
       </c>
@@ -2748,7 +3013,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>157</v>
       </c>
@@ -2756,15 +3021,15 @@
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>108</v>
       </c>
       <c r="B25" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>109</v>
       </c>
@@ -2772,7 +3037,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>140</v>
       </c>
@@ -2780,7 +3045,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>110</v>
       </c>
@@ -2788,7 +3053,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>158</v>
       </c>
@@ -2796,7 +3061,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>159</v>
       </c>

</xml_diff>

<commit_message>
actualitzant bd amb partit dia 20 de gener
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739997B9-E150-42F9-AF13-DE08FFC2C450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F041D797-7A34-A94F-B93F-2B5C8465F7C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="276">
   <si>
     <t>code_h</t>
   </si>
@@ -796,9 +796,6 @@
     <t>884933038469939200</t>
   </si>
   <si>
-    <t>E2025_217</t>
-  </si>
-  <si>
     <t>PAM</t>
   </si>
   <si>
@@ -829,25 +826,49 @@
     <t>irs_operator</t>
   </si>
   <si>
-    <t>ENDER OZBEK</t>
-  </si>
-  <si>
-    <t>SERTAC DOSTEL</t>
-  </si>
-  <si>
-    <t>CAN KUTLUATA</t>
-  </si>
-  <si>
-    <t>GIZEM UNSAL</t>
-  </si>
-  <si>
-    <t>AHMET ERKASAP</t>
-  </si>
-  <si>
-    <t>MURAT KUS</t>
-  </si>
-  <si>
     <t>1438645665340198915</t>
+  </si>
+  <si>
+    <t>U2025_147</t>
+  </si>
+  <si>
+    <t>NIN</t>
+  </si>
+  <si>
+    <t>BOU</t>
+  </si>
+  <si>
+    <t>MARC ROTHE</t>
+  </si>
+  <si>
+    <t>ALEXANDER JAHN</t>
+  </si>
+  <si>
+    <t>KIM THAMMIG</t>
+  </si>
+  <si>
+    <t>HOLGER LANGENAU</t>
+  </si>
+  <si>
+    <t>CURT KINDLER</t>
+  </si>
+  <si>
+    <t>NINERS Chemnitz</t>
+  </si>
+  <si>
+    <t>Cosea JL Bourg-en-Bresse</t>
+  </si>
+  <si>
+    <t>Chemnitz</t>
+  </si>
+  <si>
+    <t>Bourg</t>
+  </si>
+  <si>
+    <t>1414141894879084635</t>
+  </si>
+  <si>
+    <t>885149945475248149</t>
   </si>
 </sst>
 </file>
@@ -1283,8 +1304,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D24" totalsRowShown="0">
-  <autoFilter ref="A1:D24" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D26" totalsRowShown="0">
+  <autoFilter ref="A1:D26" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="4" xr3:uid="{760465A9-3097-934B-AB04-6544582DE0F4}" name="team_name"/>
@@ -1668,24 +1689,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.26953125" customWidth="1"/>
-    <col min="13" max="13" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.33203125" customWidth="1"/>
+    <col min="13" max="13" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -1708,33 +1729,33 @@
         <v>2</v>
       </c>
       <c r="H1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I1" t="s">
         <v>256</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>257</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>258</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>259</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>260</v>
       </c>
-      <c r="M1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>184</v>
+        <v>263</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="D2" s="1">
         <v>2026</v>
@@ -1743,29 +1764,27 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G2" s="1">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>267</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="M2" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1778,18 +1797,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
-  <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.1796875" customWidth="1"/>
+    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1803,7 +1822,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1817,7 +1836,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1831,7 +1850,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1845,7 +1864,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1859,7 +1878,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>141</v>
       </c>
@@ -1873,7 +1892,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>142</v>
       </c>
@@ -1887,7 +1906,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>147</v>
       </c>
@@ -1901,7 +1920,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>148</v>
       </c>
@@ -1915,7 +1934,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>160</v>
       </c>
@@ -1929,7 +1948,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>161</v>
       </c>
@@ -1943,7 +1962,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>162</v>
       </c>
@@ -1956,8 +1975,9 @@
       <c r="D12" s="4" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>163</v>
       </c>
@@ -1971,7 +1991,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>172</v>
       </c>
@@ -1985,7 +2005,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>173</v>
       </c>
@@ -1999,7 +2019,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>174</v>
       </c>
@@ -2013,7 +2033,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>175</v>
       </c>
@@ -2027,7 +2047,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>184</v>
       </c>
@@ -2038,10 +2058,10 @@
         <v>185</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>187</v>
       </c>
@@ -2055,7 +2075,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>235</v>
       </c>
@@ -2069,7 +2089,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>240</v>
       </c>
@@ -2083,7 +2103,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>243</v>
       </c>
@@ -2097,7 +2117,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>244</v>
       </c>
@@ -2111,18 +2131,46 @@
         <v>250</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>251</v>
+      </c>
+      <c r="B24" t="s">
         <v>252</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>253</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>255</v>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>263</v>
+      </c>
+      <c r="B25" t="s">
+        <v>270</v>
+      </c>
+      <c r="C25" t="s">
+        <v>272</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>264</v>
+      </c>
+      <c r="B26" t="s">
+        <v>271</v>
+      </c>
+      <c r="C26" t="s">
+        <v>273</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -2136,13 +2184,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
   <dimension ref="A1:B63"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6328125" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -2150,7 +2198,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2158,7 +2206,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2166,7 +2214,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2174,7 +2222,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2182,7 +2230,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2190,7 +2238,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2198,7 +2246,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2206,7 +2254,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2214,7 +2262,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2222,7 +2270,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2230,7 +2278,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2238,7 +2286,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -2246,7 +2294,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -2254,7 +2302,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -2262,7 +2310,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -2270,7 +2318,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -2278,7 +2326,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2286,7 +2334,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -2294,7 +2342,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -2302,7 +2350,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -2310,7 +2358,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -2318,7 +2366,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -2326,7 +2374,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -2334,7 +2382,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -2342,7 +2390,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -2350,7 +2398,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -2358,7 +2406,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -2366,7 +2414,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -2374,7 +2422,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -2382,7 +2430,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -2390,7 +2438,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>18</v>
       </c>
@@ -2398,7 +2446,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -2406,7 +2454,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -2414,7 +2462,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>18</v>
       </c>
@@ -2422,7 +2470,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>18</v>
       </c>
@@ -2430,7 +2478,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>18</v>
       </c>
@@ -2438,7 +2486,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>18</v>
       </c>
@@ -2446,7 +2494,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -2454,7 +2502,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>19</v>
       </c>
@@ -2462,7 +2510,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>19</v>
       </c>
@@ -2470,7 +2518,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>19</v>
       </c>
@@ -2478,7 +2526,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>19</v>
       </c>
@@ -2486,7 +2534,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -2494,7 +2542,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>19</v>
       </c>
@@ -2502,7 +2550,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -2510,7 +2558,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -2518,7 +2566,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>19</v>
       </c>
@@ -2526,7 +2574,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>19</v>
       </c>
@@ -2534,7 +2582,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>19</v>
       </c>
@@ -2542,7 +2590,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>19</v>
       </c>
@@ -2550,7 +2598,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -2558,7 +2606,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>19</v>
       </c>
@@ -2566,7 +2614,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>172</v>
       </c>
@@ -2574,7 +2622,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>172</v>
       </c>
@@ -2582,7 +2630,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>172</v>
       </c>
@@ -2590,7 +2638,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>172</v>
       </c>
@@ -2598,7 +2646,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>172</v>
       </c>
@@ -2606,7 +2654,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>172</v>
       </c>
@@ -2614,7 +2662,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>172</v>
       </c>
@@ -2622,7 +2670,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>172</v>
       </c>
@@ -2630,7 +2678,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>172</v>
       </c>
@@ -2638,7 +2686,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>172</v>
       </c>
@@ -2657,13 +2705,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
-    <col min="2" max="2" width="26.36328125" customWidth="1"/>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -2671,7 +2719,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>226</v>
       </c>
@@ -2679,7 +2727,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>227</v>
       </c>
@@ -2687,7 +2735,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>228</v>
       </c>
@@ -2695,7 +2743,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>229</v>
       </c>
@@ -2703,7 +2751,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>230</v>
       </c>
@@ -2711,7 +2759,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>231</v>
       </c>
@@ -2719,7 +2767,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>232</v>
       </c>
@@ -2727,7 +2775,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>233</v>
       </c>
@@ -2735,7 +2783,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>234</v>
       </c>
@@ -2754,24 +2802,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2823,13 +2871,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E819B3A5-8F6D-6649-8C82-B76A24B61AC2}">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>90</v>
       </c>
@@ -2837,7 +2885,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -2845,7 +2893,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>92</v>
       </c>
@@ -2853,7 +2901,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -2861,7 +2909,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -2869,7 +2917,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -2877,7 +2925,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -2885,7 +2933,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>154</v>
       </c>
@@ -2893,7 +2941,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -2901,7 +2949,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>98</v>
       </c>
@@ -2909,7 +2957,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>99</v>
       </c>
@@ -2917,7 +2965,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>100</v>
       </c>
@@ -2925,7 +2973,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>101</v>
       </c>
@@ -2933,7 +2981,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>102</v>
       </c>
@@ -2941,7 +2989,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>103</v>
       </c>
@@ -2949,7 +2997,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>104</v>
       </c>
@@ -2957,7 +3005,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>155</v>
       </c>
@@ -2965,7 +3013,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>105</v>
       </c>
@@ -2973,7 +3021,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -2981,7 +3029,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>107</v>
       </c>
@@ -2989,7 +3037,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -2997,7 +3045,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>126</v>
       </c>
@@ -3005,7 +3053,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>156</v>
       </c>
@@ -3013,7 +3061,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>157</v>
       </c>
@@ -3021,7 +3069,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>108</v>
       </c>
@@ -3029,7 +3077,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>109</v>
       </c>
@@ -3037,7 +3085,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>140</v>
       </c>
@@ -3045,7 +3093,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>110</v>
       </c>
@@ -3053,7 +3101,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>158</v>
       </c>
@@ -3061,7 +3109,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>159</v>
       </c>

</xml_diff>

<commit_message>
actualitzacio bd 20 gener
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F041D797-7A34-A94F-B93F-2B5C8465F7C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E64C555-48E0-4A32-BD04-B1F43E3EDB11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -904,7 +904,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -951,11 +951,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -967,6 +980,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1689,24 +1703,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.33203125" customWidth="1"/>
-    <col min="13" max="13" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -1747,7 +1761,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>262</v>
       </c>
@@ -1770,13 +1784,13 @@
         <v>15</v>
       </c>
       <c r="H2" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>266</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>267</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>268</v>
@@ -1798,17 +1812,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
   <dimension ref="A1:I26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.1640625" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -1822,7 +1836,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1836,7 +1850,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1850,7 +1864,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1864,7 +1878,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1878,7 +1892,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>141</v>
       </c>
@@ -1892,7 +1906,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>142</v>
       </c>
@@ -1906,7 +1920,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>147</v>
       </c>
@@ -1920,7 +1934,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>148</v>
       </c>
@@ -1934,7 +1948,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>160</v>
       </c>
@@ -1948,7 +1962,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>161</v>
       </c>
@@ -1962,7 +1976,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>162</v>
       </c>
@@ -1977,7 +1991,7 @@
       </c>
       <c r="I12" s="3"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>163</v>
       </c>
@@ -1991,7 +2005,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>172</v>
       </c>
@@ -2005,7 +2019,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>173</v>
       </c>
@@ -2019,7 +2033,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>174</v>
       </c>
@@ -2033,7 +2047,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>175</v>
       </c>
@@ -2047,7 +2061,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>184</v>
       </c>
@@ -2061,7 +2075,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>187</v>
       </c>
@@ -2075,7 +2089,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>235</v>
       </c>
@@ -2089,7 +2103,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>240</v>
       </c>
@@ -2103,7 +2117,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>243</v>
       </c>
@@ -2117,7 +2131,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>244</v>
       </c>
@@ -2131,7 +2145,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>251</v>
       </c>
@@ -2145,7 +2159,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>263</v>
       </c>
@@ -2159,7 +2173,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>264</v>
       </c>
@@ -2184,13 +2198,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42514417-67C5-4950-98C4-A0D6E48593E8}">
   <dimension ref="A1:B63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -2198,7 +2212,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2206,7 +2220,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2214,7 +2228,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2222,7 +2236,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2230,7 +2244,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2238,7 +2252,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2246,7 +2260,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2254,7 +2268,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2262,7 +2276,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2270,7 +2284,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2278,7 +2292,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2286,7 +2300,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -2294,7 +2308,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -2302,7 +2316,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -2310,7 +2324,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -2318,7 +2332,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -2326,7 +2340,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2334,7 +2348,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -2342,7 +2356,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -2350,7 +2364,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -2358,7 +2372,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -2366,7 +2380,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -2374,7 +2388,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -2382,7 +2396,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -2390,7 +2404,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -2398,7 +2412,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -2406,7 +2420,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -2414,7 +2428,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -2422,7 +2436,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -2430,7 +2444,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -2438,7 +2452,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>18</v>
       </c>
@@ -2446,7 +2460,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -2454,7 +2468,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>18</v>
       </c>
@@ -2462,7 +2476,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>18</v>
       </c>
@@ -2470,7 +2484,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>18</v>
       </c>
@@ -2478,7 +2492,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>18</v>
       </c>
@@ -2486,7 +2500,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>18</v>
       </c>
@@ -2494,7 +2508,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -2502,7 +2516,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>19</v>
       </c>
@@ -2510,7 +2524,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>19</v>
       </c>
@@ -2518,7 +2532,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>19</v>
       </c>
@@ -2526,7 +2540,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>19</v>
       </c>
@@ -2534,7 +2548,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -2542,7 +2556,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>19</v>
       </c>
@@ -2550,7 +2564,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>19</v>
       </c>
@@ -2558,7 +2572,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>19</v>
       </c>
@@ -2566,7 +2580,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>19</v>
       </c>
@@ -2574,7 +2588,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>19</v>
       </c>
@@ -2582,7 +2596,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>19</v>
       </c>
@@ -2590,7 +2604,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>19</v>
       </c>
@@ -2598,7 +2612,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>19</v>
       </c>
@@ -2606,7 +2620,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>19</v>
       </c>
@@ -2614,7 +2628,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="54" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>172</v>
       </c>
@@ -2622,7 +2636,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>172</v>
       </c>
@@ -2630,7 +2644,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>172</v>
       </c>
@@ -2638,7 +2652,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>172</v>
       </c>
@@ -2646,7 +2660,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>172</v>
       </c>
@@ -2654,7 +2668,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>172</v>
       </c>
@@ -2662,7 +2676,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>172</v>
       </c>
@@ -2670,7 +2684,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>172</v>
       </c>
@@ -2678,7 +2692,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>172</v>
       </c>
@@ -2686,7 +2700,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>172</v>
       </c>
@@ -2705,13 +2719,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C876E4A3-D4DE-42E2-AC32-9D34F376F8C4}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -2719,7 +2733,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>226</v>
       </c>
@@ -2727,7 +2741,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>227</v>
       </c>
@@ -2735,7 +2749,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>228</v>
       </c>
@@ -2743,7 +2757,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>229</v>
       </c>
@@ -2751,7 +2765,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>230</v>
       </c>
@@ -2759,7 +2773,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>231</v>
       </c>
@@ -2767,7 +2781,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>232</v>
       </c>
@@ -2775,7 +2789,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>233</v>
       </c>
@@ -2783,7 +2797,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>234</v>
       </c>
@@ -2802,24 +2816,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A863807A-0BDA-4D42-BA31-A09BFCF72226}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2871,13 +2885,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E819B3A5-8F6D-6649-8C82-B76A24B61AC2}">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>90</v>
       </c>
@@ -2885,7 +2899,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -2893,7 +2907,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>92</v>
       </c>
@@ -2901,7 +2915,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -2909,7 +2923,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -2917,7 +2931,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -2925,7 +2939,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>96</v>
       </c>
@@ -2933,7 +2947,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>154</v>
       </c>
@@ -2941,7 +2955,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>97</v>
       </c>
@@ -2949,7 +2963,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>98</v>
       </c>
@@ -2957,7 +2971,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>99</v>
       </c>
@@ -2965,7 +2979,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>100</v>
       </c>
@@ -2973,7 +2987,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>101</v>
       </c>
@@ -2981,7 +2995,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>102</v>
       </c>
@@ -2989,7 +3003,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>103</v>
       </c>
@@ -2997,7 +3011,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>104</v>
       </c>
@@ -3005,7 +3019,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>155</v>
       </c>
@@ -3013,7 +3027,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>105</v>
       </c>
@@ -3021,7 +3035,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -3029,7 +3043,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>107</v>
       </c>
@@ -3037,7 +3051,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>128</v>
       </c>
@@ -3045,7 +3059,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>126</v>
       </c>
@@ -3053,7 +3067,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>156</v>
       </c>
@@ -3061,7 +3075,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>157</v>
       </c>
@@ -3069,7 +3083,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>108</v>
       </c>
@@ -3077,7 +3091,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>109</v>
       </c>
@@ -3085,7 +3099,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>140</v>
       </c>
@@ -3093,7 +3107,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>110</v>
       </c>
@@ -3101,7 +3115,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>158</v>
       </c>
@@ -3109,7 +3123,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>159</v>
       </c>

</xml_diff>

<commit_message>
dades 21 de gener
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E64C555-48E0-4A32-BD04-B1F43E3EDB11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A228BF3-7920-4284-98F1-4C9B412B0168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="279">
   <si>
     <t>code_h</t>
   </si>
@@ -829,30 +829,12 @@
     <t>1438645665340198915</t>
   </si>
   <si>
-    <t>U2025_147</t>
-  </si>
-  <si>
     <t>NIN</t>
   </si>
   <si>
     <t>BOU</t>
   </si>
   <si>
-    <t>MARC ROTHE</t>
-  </si>
-  <si>
-    <t>ALEXANDER JAHN</t>
-  </si>
-  <si>
-    <t>KIM THAMMIG</t>
-  </si>
-  <si>
-    <t>HOLGER LANGENAU</t>
-  </si>
-  <si>
-    <t>CURT KINDLER</t>
-  </si>
-  <si>
     <t>NINERS Chemnitz</t>
   </si>
   <si>
@@ -869,6 +851,33 @@
   </si>
   <si>
     <t>885149945475248149</t>
+  </si>
+  <si>
+    <t>U2025_148</t>
+  </si>
+  <si>
+    <t>BUD</t>
+  </si>
+  <si>
+    <t>Buducnost VOLI Podgorica</t>
+  </si>
+  <si>
+    <t>885149103577772093</t>
+  </si>
+  <si>
+    <t>MAN</t>
+  </si>
+  <si>
+    <t>BAXI Manresa</t>
+  </si>
+  <si>
+    <t>1414140640052248658</t>
+  </si>
+  <si>
+    <t>Buducnost</t>
+  </si>
+  <si>
+    <t>Manresa</t>
   </si>
 </sst>
 </file>
@@ -1318,8 +1327,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D26" totalsRowShown="0">
-  <autoFilter ref="A1:D26" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D28" totalsRowShown="0">
+  <autoFilter ref="A1:D28" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="4" xr3:uid="{760465A9-3097-934B-AB04-6544582DE0F4}" name="team_name"/>
@@ -1763,13 +1772,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>263</v>
+        <v>160</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="D2" s="1">
         <v>2026</v>
@@ -1778,26 +1787,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="1">
         <v>15</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>269</v>
-      </c>
+      <c r="H2" s="8"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
       <c r="M2" s="8"/>
     </row>
   </sheetData>
@@ -1811,7 +1810,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
@@ -2161,30 +2160,58 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B25" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="C25" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B26" t="s">
+        <v>265</v>
+      </c>
+      <c r="C26" t="s">
+        <v>267</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>271</v>
       </c>
-      <c r="C26" t="s">
+      <c r="B27" t="s">
+        <v>272</v>
+      </c>
+      <c r="C27" t="s">
+        <v>277</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="D26" s="4" t="s">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>274</v>
+      </c>
+      <c r="B28" t="s">
         <v>275</v>
+      </c>
+      <c r="C28" t="s">
+        <v>278</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dia 22 i 23 de gener
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A228BF3-7920-4284-98F1-4C9B412B0168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25221259-776A-476C-A39D-F1C6C4B06774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="288">
   <si>
     <t>code_h</t>
   </si>
@@ -853,9 +853,6 @@
     <t>885149945475248149</t>
   </si>
   <si>
-    <t>U2025_148</t>
-  </si>
-  <si>
     <t>BUD</t>
   </si>
   <si>
@@ -878,6 +875,36 @@
   </si>
   <si>
     <t>Manresa</t>
+  </si>
+  <si>
+    <t>E2025_231</t>
+  </si>
+  <si>
+    <t>OLY</t>
+  </si>
+  <si>
+    <t>E2025_235</t>
+  </si>
+  <si>
+    <t>MCO</t>
+  </si>
+  <si>
+    <t>AS Monaco</t>
+  </si>
+  <si>
+    <t>Olympiacos Piraeus</t>
+  </si>
+  <si>
+    <t>884934311583809536</t>
+  </si>
+  <si>
+    <t>884932778553139230</t>
+  </si>
+  <si>
+    <t>Olympiacos</t>
+  </si>
+  <si>
+    <t>Monaco</t>
   </si>
 </sst>
 </file>
@@ -977,7 +1004,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -990,6 +1017,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1302,8 +1330,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:M2" totalsRowShown="0">
-  <autoFilter ref="A1:M2" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:M3" totalsRowShown="0">
+  <autoFilter ref="A1:M3" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G2">
     <sortCondition ref="F1:F2"/>
   </sortState>
@@ -1327,8 +1355,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D28" totalsRowShown="0">
-  <autoFilter ref="A1:D28" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D30" totalsRowShown="0">
+  <autoFilter ref="A1:D30" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="4" xr3:uid="{760465A9-3097-934B-AB04-6544582DE0F4}" name="team_name"/>
@@ -1711,7 +1739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
@@ -1772,13 +1800,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>160</v>
+        <v>243</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="D2" s="1">
         <v>2026</v>
@@ -1787,10 +1815,10 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" s="1">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="9"/>
@@ -1798,6 +1826,35 @@
       <c r="K2" s="8"/>
       <c r="L2" s="8"/>
       <c r="M2" s="8"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" s="9">
+        <v>2026</v>
+      </c>
+      <c r="E3" s="9">
+        <v>1</v>
+      </c>
+      <c r="F3" s="9">
+        <v>22</v>
+      </c>
+      <c r="G3" s="9">
+        <v>24</v>
+      </c>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1810,7 +1867,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
@@ -2188,30 +2245,58 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>270</v>
+      </c>
+      <c r="B27" t="s">
         <v>271</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
+        <v>276</v>
+      </c>
+      <c r="D27" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="C27" t="s">
-        <v>277</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>273</v>
+      </c>
+      <c r="B28" t="s">
         <v>274</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
+        <v>277</v>
+      </c>
+      <c r="D28" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="C28" t="s">
-        <v>278</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>276</v>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>279</v>
+      </c>
+      <c r="B29" t="s">
+        <v>283</v>
+      </c>
+      <c r="C29" t="s">
+        <v>286</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>281</v>
+      </c>
+      <c r="B30" t="s">
+        <v>282</v>
+      </c>
+      <c r="C30" t="s">
+        <v>287</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
canvis a base de dades amb partits de setmana 27-30 de gener
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25221259-776A-476C-A39D-F1C6C4B06774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA63633-F4B8-49CF-8B1D-97DDC9203948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="314">
   <si>
     <t>code_h</t>
   </si>
@@ -877,15 +877,9 @@
     <t>Manresa</t>
   </si>
   <si>
-    <t>E2025_231</t>
-  </si>
-  <si>
     <t>OLY</t>
   </si>
   <si>
-    <t>E2025_235</t>
-  </si>
-  <si>
     <t>MCO</t>
   </si>
   <si>
@@ -905,6 +899,90 @@
   </si>
   <si>
     <t>Monaco</t>
+  </si>
+  <si>
+    <t>U2025_158</t>
+  </si>
+  <si>
+    <t>U2025_160</t>
+  </si>
+  <si>
+    <t>E2025_246</t>
+  </si>
+  <si>
+    <t>Partizan Mozzart Bet Belgrade</t>
+  </si>
+  <si>
+    <t>Partizan</t>
+  </si>
+  <si>
+    <t>PAR</t>
+  </si>
+  <si>
+    <t>885150446631682078</t>
+  </si>
+  <si>
+    <t>SILVIA BOTTURA</t>
+  </si>
+  <si>
+    <t>SASHA ZORDAN</t>
+  </si>
+  <si>
+    <t>TOMMASO MOLO</t>
+  </si>
+  <si>
+    <t>FJORENCO HYSI</t>
+  </si>
+  <si>
+    <t>GUILLAUME VORS</t>
+  </si>
+  <si>
+    <t>MAXIME VASSELIN</t>
+  </si>
+  <si>
+    <t>SOFYAN LANGER</t>
+  </si>
+  <si>
+    <t>NOEMI DEIMICHEL</t>
+  </si>
+  <si>
+    <t>MAXIME JANNON</t>
+  </si>
+  <si>
+    <t>ARNAUD WEICKERT</t>
+  </si>
+  <si>
+    <t>ALESSANDRO ZUCCA</t>
+  </si>
+  <si>
+    <t>RENATO BOCCOTTI</t>
+  </si>
+  <si>
+    <t>EMANUELA DALLA COSTA</t>
+  </si>
+  <si>
+    <t>SIMONE VLACHOS</t>
+  </si>
+  <si>
+    <t>CINZIA COZZI</t>
+  </si>
+  <si>
+    <t>ENRICO ROSTI</t>
+  </si>
+  <si>
+    <t>E2025_247</t>
+  </si>
+  <si>
+    <t>Virtus Bologna</t>
+  </si>
+  <si>
+    <t>885903947624247337</t>
+  </si>
+  <si>
+    <t>VIR</t>
+  </si>
+  <si>
+    <t>Virtus</t>
   </si>
 </sst>
 </file>
@@ -940,7 +1018,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1000,11 +1078,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1018,6 +1109,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1330,8 +1422,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:M3" totalsRowShown="0">
-  <autoFilter ref="A1:M3" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}" name="Table1" displayName="Table1" ref="A1:M5" totalsRowShown="0">
+  <autoFilter ref="A1:M5" xr:uid="{37375DB6-3E3F-4BC0-A810-F73B4F912A87}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G2">
     <sortCondition ref="F1:F2"/>
   </sortState>
@@ -1355,8 +1447,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D30" totalsRowShown="0">
-  <autoFilter ref="A1:D30" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}" name="Table2" displayName="Table2" ref="A1:D32" totalsRowShown="0">
+  <autoFilter ref="A1:D32" xr:uid="{E1ACAC3A-2FB2-44B6-A0CB-4E2ECC44CF7A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{11EC5321-3796-441B-BC0C-81CBCDF2EA1A}" name="team_code"/>
     <tableColumn id="4" xr3:uid="{760465A9-3097-934B-AB04-6544582DE0F4}" name="team_name"/>
@@ -1739,22 +1831,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5C88AB7-F763-4FF2-AF91-9177F25C5745}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.08984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
@@ -1800,13 +1892,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>243</v>
+        <v>173</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>279</v>
+        <v>160</v>
       </c>
       <c r="D2" s="1">
         <v>2026</v>
@@ -1815,27 +1907,35 @@
         <v>1</v>
       </c>
       <c r="F2" s="1">
-        <v>22</v>
-      </c>
-      <c r="G2" s="1">
-        <v>24</v>
-      </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+        <v>27</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>300</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="M2" s="11"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>147</v>
+        <v>263</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>281</v>
+        <v>161</v>
       </c>
       <c r="D3" s="9">
         <v>2026</v>
@@ -1844,17 +1944,91 @@
         <v>1</v>
       </c>
       <c r="F3" s="9">
-        <v>22</v>
-      </c>
-      <c r="G3" s="9">
-        <v>24</v>
-      </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
+        <v>28</v>
+      </c>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>302</v>
+      </c>
       <c r="M3" s="9"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="D4" s="9">
+        <v>2026</v>
+      </c>
+      <c r="E4" s="9">
+        <v>1</v>
+      </c>
+      <c r="F4" s="9">
+        <v>29</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="D5" s="9">
+        <v>2026</v>
+      </c>
+      <c r="E5" s="9">
+        <v>1</v>
+      </c>
+      <c r="F5" s="9">
+        <v>30</v>
+      </c>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1867,7 +2041,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46F5EBAB-4F91-44CC-8DBB-AB55169F26CC}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
@@ -2273,30 +2447,58 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B29" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C29" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B30" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C30" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>291</v>
+      </c>
+      <c r="B31" t="s">
+        <v>289</v>
+      </c>
+      <c r="C31" t="s">
+        <v>290</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>312</v>
+      </c>
+      <c r="B32" t="s">
+        <v>310</v>
+      </c>
+      <c r="C32" t="s">
+        <v>313</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualització base dades partit dia 30 de gener
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA63633-F4B8-49CF-8B1D-97DDC9203948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB54CAB3-EDE5-4C99-A2A5-A32831BB0E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
+    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{ACA68719-90DF-4854-9EF3-E6278E5C527A}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="320">
   <si>
     <t>code_h</t>
   </si>
@@ -983,6 +983,24 @@
   </si>
   <si>
     <t>Virtus</t>
+  </si>
+  <si>
+    <t>CATHERINE RICARD</t>
+  </si>
+  <si>
+    <t>VANESSA CAUCHIE</t>
+  </si>
+  <si>
+    <t>CLAUDINE CARADONNA</t>
+  </si>
+  <si>
+    <t>JEAN-PAUL JUSTINIANO</t>
+  </si>
+  <si>
+    <t>THIERRY GACHE</t>
+  </si>
+  <si>
+    <t>DAVID MARTINOTTI</t>
   </si>
 </sst>
 </file>
@@ -1844,9 +1862,8 @@
     <col min="8" max="8" width="18.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16.90625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
@@ -2023,12 +2040,24 @@
         <v>30</v>
       </c>
       <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
+      <c r="H5" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>319</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
millores en l'estructura del backend relacionat amb la generació del report
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2C71B5-873C-944E-B617-77B86058369D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2BC1321-5429-3C4C-8EAD-F3F78ED05646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="374">
   <si>
     <t>game_code</t>
   </si>
@@ -1111,13 +1111,49 @@
   </si>
   <si>
     <t>1414142141256437923</t>
+  </si>
+  <si>
+    <t>ORHAN YENIHAYAT</t>
+  </si>
+  <si>
+    <t>KEREM SIRMAGIL</t>
+  </si>
+  <si>
+    <t>CAN KUTLUATA</t>
+  </si>
+  <si>
+    <t>AHMET YILDIZ</t>
+  </si>
+  <si>
+    <t>MERVE SAGLAM</t>
+  </si>
+  <si>
+    <t>MURAT KUS</t>
+  </si>
+  <si>
+    <t>SEBASTIAN BLANZ</t>
+  </si>
+  <si>
+    <t>MANUEL HERZOG</t>
+  </si>
+  <si>
+    <t>FELIX ROEHLICH</t>
+  </si>
+  <si>
+    <t>ANDREAS GREPPMAYR</t>
+  </si>
+  <si>
+    <t>ROBERT BAYERER</t>
+  </si>
+  <si>
+    <t>ROBERT TAVASZI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1135,6 +1171,12 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1185,7 +1227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
@@ -1197,6 +1239,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1861,6 +1904,24 @@
       <c r="G6">
         <v>26</v>
       </c>
+      <c r="H6" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>367</v>
+      </c>
       <c r="N6" t="b">
         <v>0</v>
       </c>
@@ -1886,6 +1947,24 @@
       </c>
       <c r="G7">
         <v>26</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>373</v>
       </c>
       <c r="N7" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
millora en rapidesa a l'hora d'extreure els threads d'un canal de discord
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eloiverge/Projects/reports-automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloi.verge\Projects\reports-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2BC1321-5429-3C4C-8EAD-F3F78ED05646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A729A3-CBDD-456B-8E8F-F8BFD2087050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" r:id="rId1"/>
@@ -171,6 +171,84 @@
     <t>DAVID MARTINOTTI</t>
   </si>
   <si>
+    <t>E2025_251</t>
+  </si>
+  <si>
+    <t>IST</t>
+  </si>
+  <si>
+    <t>PAM</t>
+  </si>
+  <si>
+    <t>CAN KUTLUATA</t>
+  </si>
+  <si>
+    <t>ORHAN YENIHAYAT</t>
+  </si>
+  <si>
+    <t>KEREM SIRMAGIL</t>
+  </si>
+  <si>
+    <t>AHMET YILDIZ</t>
+  </si>
+  <si>
+    <t>MERVE SAGLAM</t>
+  </si>
+  <si>
+    <t>MURAT KUS</t>
+  </si>
+  <si>
+    <t>E2025_256</t>
+  </si>
+  <si>
+    <t>MUN</t>
+  </si>
+  <si>
+    <t>PRS</t>
+  </si>
+  <si>
+    <t>SEBASTIAN BLANZ</t>
+  </si>
+  <si>
+    <t>MANUEL HERZOG</t>
+  </si>
+  <si>
+    <t>FELIX ROEHLICH</t>
+  </si>
+  <si>
+    <t>ANDREAS GREPPMAYR</t>
+  </si>
+  <si>
+    <t>ROBERT BAYERER</t>
+  </si>
+  <si>
+    <t>ROBERT TAVASZI</t>
+  </si>
+  <si>
+    <t>E2025_260</t>
+  </si>
+  <si>
+    <t>ASV</t>
+  </si>
+  <si>
+    <t>U2025_165</t>
+  </si>
+  <si>
+    <t>HAM</t>
+  </si>
+  <si>
+    <t>LJU</t>
+  </si>
+  <si>
+    <t>E2025_268</t>
+  </si>
+  <si>
+    <t>RED</t>
+  </si>
+  <si>
+    <t>TEL</t>
+  </si>
+  <si>
     <t>team_code</t>
   </si>
   <si>
@@ -183,9 +261,6 @@
     <t>discord_channel_id</t>
   </si>
   <si>
-    <t>PRS</t>
-  </si>
-  <si>
     <t>Paris Basketball</t>
   </si>
   <si>
@@ -207,9 +282,6 @@
     <t>884933776889749504</t>
   </si>
   <si>
-    <t>LJU</t>
-  </si>
-  <si>
     <t>Cedevita Olimpija Ljubljana</t>
   </si>
   <si>
@@ -375,9 +447,6 @@
     <t>1438645665340198915</t>
   </si>
   <si>
-    <t>RED</t>
-  </si>
-  <si>
     <t>Crvena Zvezda Meridianbet Belgrade</t>
   </si>
   <si>
@@ -411,9 +480,6 @@
     <t>1144317098089263114</t>
   </si>
   <si>
-    <t>IST</t>
-  </si>
-  <si>
     <t>Anadolu Efes Istanbul</t>
   </si>
   <si>
@@ -435,9 +501,6 @@
     <t>884933038469939200</t>
   </si>
   <si>
-    <t>PAM</t>
-  </si>
-  <si>
     <t>Valencia Basket</t>
   </si>
   <si>
@@ -531,6 +594,102 @@
     <t>885903947624247337</t>
   </si>
   <si>
+    <t>FC Bayern Munich</t>
+  </si>
+  <si>
+    <t>Bayern</t>
+  </si>
+  <si>
+    <t>884933903222186024</t>
+  </si>
+  <si>
+    <t>LDLC ASVEL Villeurbanne</t>
+  </si>
+  <si>
+    <t>ASVEL</t>
+  </si>
+  <si>
+    <t>884934113176477726</t>
+  </si>
+  <si>
+    <t>Maccabi Rapyd Tel Aviv</t>
+  </si>
+  <si>
+    <t>Maccabi</t>
+  </si>
+  <si>
+    <t>884934195707781182</t>
+  </si>
+  <si>
+    <t>Veolia Towers Hamburg</t>
+  </si>
+  <si>
+    <t>Hamburg</t>
+  </si>
+  <si>
+    <t>885149528041328690</t>
+  </si>
+  <si>
+    <t>BAH</t>
+  </si>
+  <si>
+    <t>Bahcesehir College Istanbul</t>
+  </si>
+  <si>
+    <t>Bahcesehir</t>
+  </si>
+  <si>
+    <t>1287802616687890484</t>
+  </si>
+  <si>
+    <t>LKB</t>
+  </si>
+  <si>
+    <t>Lietkabelis Panevezys</t>
+  </si>
+  <si>
+    <t>Lietkabelis</t>
+  </si>
+  <si>
+    <t>885149715501580358</t>
+  </si>
+  <si>
+    <t>LLI</t>
+  </si>
+  <si>
+    <t>London Lions</t>
+  </si>
+  <si>
+    <t>London</t>
+  </si>
+  <si>
+    <t>1414141685822394399</t>
+  </si>
+  <si>
+    <t>NIO</t>
+  </si>
+  <si>
+    <t>Panionios Cosmorama Travel Athens</t>
+  </si>
+  <si>
+    <t>Panionios</t>
+  </si>
+  <si>
+    <t>1414141990165287043</t>
+  </si>
+  <si>
+    <t>WRO</t>
+  </si>
+  <si>
+    <t>Slask Wroclaw</t>
+  </si>
+  <si>
+    <t>Slask</t>
+  </si>
+  <si>
+    <t>1414142141256437923</t>
+  </si>
+  <si>
     <t>name</t>
   </si>
   <si>
@@ -988,172 +1147,13 @@
   </si>
   <si>
     <t>Throw In Foul</t>
-  </si>
-  <si>
-    <t>E2025_251</t>
-  </si>
-  <si>
-    <t>E2025_256</t>
-  </si>
-  <si>
-    <t>U2025_165</t>
-  </si>
-  <si>
-    <t>E2025_260</t>
-  </si>
-  <si>
-    <t>E2025_268</t>
-  </si>
-  <si>
-    <t>MUN</t>
-  </si>
-  <si>
-    <t>FC Bayern Munich</t>
-  </si>
-  <si>
-    <t>ASV</t>
-  </si>
-  <si>
-    <t>LDLC ASVEL Villeurbanne</t>
-  </si>
-  <si>
-    <t>TEL</t>
-  </si>
-  <si>
-    <t>Maccabi Rapyd Tel Aviv</t>
-  </si>
-  <si>
-    <t>HAM</t>
-  </si>
-  <si>
-    <t>Veolia Towers Hamburg</t>
-  </si>
-  <si>
-    <t>Bayern</t>
-  </si>
-  <si>
-    <t>ASVEL</t>
-  </si>
-  <si>
-    <t>Maccabi</t>
-  </si>
-  <si>
-    <t>Hamburg</t>
-  </si>
-  <si>
-    <t>884933903222186024</t>
-  </si>
-  <si>
-    <t>884934113176477726</t>
-  </si>
-  <si>
-    <t>884934195707781182</t>
-  </si>
-  <si>
-    <t>885149528041328690</t>
-  </si>
-  <si>
-    <t>BAH</t>
-  </si>
-  <si>
-    <t>Bahcesehir College Istanbul</t>
-  </si>
-  <si>
-    <t>LKB</t>
-  </si>
-  <si>
-    <t>Lietkabelis Panevezys</t>
-  </si>
-  <si>
-    <t>LLI</t>
-  </si>
-  <si>
-    <t>London Lions</t>
-  </si>
-  <si>
-    <t>NIO</t>
-  </si>
-  <si>
-    <t>Panionios Cosmorama Travel Athens</t>
-  </si>
-  <si>
-    <t>WRO</t>
-  </si>
-  <si>
-    <t>Slask Wroclaw</t>
-  </si>
-  <si>
-    <t>Bahcesehir</t>
-  </si>
-  <si>
-    <t>Lietkabelis</t>
-  </si>
-  <si>
-    <t>London</t>
-  </si>
-  <si>
-    <t>Panionios</t>
-  </si>
-  <si>
-    <t>Slask</t>
-  </si>
-  <si>
-    <t>1287802616687890484</t>
-  </si>
-  <si>
-    <t>885149715501580358</t>
-  </si>
-  <si>
-    <t>1414141685822394399</t>
-  </si>
-  <si>
-    <t>1414141990165287043</t>
-  </si>
-  <si>
-    <t>1414142141256437923</t>
-  </si>
-  <si>
-    <t>ORHAN YENIHAYAT</t>
-  </si>
-  <si>
-    <t>KEREM SIRMAGIL</t>
-  </si>
-  <si>
-    <t>CAN KUTLUATA</t>
-  </si>
-  <si>
-    <t>AHMET YILDIZ</t>
-  </si>
-  <si>
-    <t>MERVE SAGLAM</t>
-  </si>
-  <si>
-    <t>MURAT KUS</t>
-  </si>
-  <si>
-    <t>SEBASTIAN BLANZ</t>
-  </si>
-  <si>
-    <t>MANUEL HERZOG</t>
-  </si>
-  <si>
-    <t>FELIX ROEHLICH</t>
-  </si>
-  <si>
-    <t>ANDREAS GREPPMAYR</t>
-  </si>
-  <si>
-    <t>ROBERT BAYERER</t>
-  </si>
-  <si>
-    <t>ROBERT TAVASZI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1171,12 +1171,6 @@
       <b/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1227,7 +1221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
@@ -1239,7 +1233,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1650,25 +1643,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.33203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1712,7 +1689,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1753,7 +1730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1794,7 +1771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1838,7 +1815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -1882,15 +1859,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>321</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>136</v>
+        <v>50</v>
       </c>
       <c r="D6">
         <v>2026</v>
@@ -1904,37 +1881,37 @@
       <c r="G6">
         <v>26</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>363</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>365</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>366</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>367</v>
+      <c r="H6" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" t="s">
+        <v>53</v>
+      </c>
+      <c r="K6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" t="s">
+        <v>56</v>
       </c>
       <c r="N6" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>322</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>326</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D7">
         <v>2026</v>
@@ -1948,37 +1925,37 @@
       <c r="G7">
         <v>26</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>368</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>369</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>370</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>371</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>372</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>373</v>
+      <c r="H7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" t="s">
+        <v>61</v>
+      </c>
+      <c r="J7" t="s">
+        <v>62</v>
+      </c>
+      <c r="K7" t="s">
+        <v>63</v>
+      </c>
+      <c r="L7" t="s">
+        <v>64</v>
+      </c>
+      <c r="M7" t="s">
+        <v>65</v>
       </c>
       <c r="N7" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>324</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>328</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>2026</v>
@@ -1996,15 +1973,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>323</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>332</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D9">
         <v>2026</v>
@@ -2022,15 +1999,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>325</v>
+        <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="C10" t="s">
-        <v>330</v>
+        <v>73</v>
       </c>
       <c r="D10">
         <v>2026</v>
@@ -2056,589 +2033,589 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="45.1640625" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="C14" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="C16" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="B18" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>144</v>
       </c>
       <c r="C20" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>124</v>
+        <v>147</v>
       </c>
       <c r="B21" t="s">
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="C21" t="s">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>128</v>
+        <v>49</v>
       </c>
       <c r="B22" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="C22" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="B23" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="C23" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>136</v>
+        <v>50</v>
       </c>
       <c r="B24" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="C24" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="B25" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="C25" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
       <c r="B26" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="C26" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="B27" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="C27" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B28" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C28" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="B29" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="C29" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="C30" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="C31" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="C32" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>326</v>
+        <v>58</v>
       </c>
       <c r="B33" t="s">
-        <v>327</v>
+        <v>189</v>
       </c>
       <c r="C33" t="s">
-        <v>334</v>
+        <v>190</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>328</v>
+        <v>67</v>
       </c>
       <c r="B34" t="s">
-        <v>329</v>
+        <v>192</v>
       </c>
       <c r="C34" t="s">
-        <v>335</v>
+        <v>193</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>330</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>331</v>
+        <v>195</v>
       </c>
       <c r="C35" t="s">
-        <v>336</v>
+        <v>196</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>332</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>333</v>
+        <v>198</v>
       </c>
       <c r="C36" t="s">
-        <v>337</v>
+        <v>199</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>342</v>
+        <v>201</v>
       </c>
       <c r="B37" t="s">
-        <v>343</v>
+        <v>202</v>
       </c>
       <c r="C37" t="s">
-        <v>352</v>
+        <v>203</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>344</v>
+        <v>205</v>
       </c>
       <c r="B38" t="s">
-        <v>345</v>
+        <v>206</v>
       </c>
       <c r="C38" t="s">
-        <v>353</v>
+        <v>207</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>346</v>
+        <v>209</v>
       </c>
       <c r="B39" t="s">
-        <v>347</v>
+        <v>210</v>
       </c>
       <c r="C39" t="s">
-        <v>354</v>
+        <v>211</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>348</v>
+        <v>213</v>
       </c>
       <c r="B40" t="s">
-        <v>349</v>
+        <v>214</v>
       </c>
       <c r="C40" t="s">
-        <v>355</v>
+        <v>215</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>350</v>
+        <v>217</v>
       </c>
       <c r="B41" t="s">
-        <v>351</v>
+        <v>218</v>
       </c>
       <c r="C41" t="s">
-        <v>356</v>
+        <v>219</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>361</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -2652,514 +2629,514 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B15" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B16" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B17" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B18" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B22" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B23" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B24" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="B25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B27" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B28" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B29" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B30" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B31" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B34" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B36" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B37" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="B38" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B55" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B56" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B57" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B58" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B59" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B60" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B61" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B62" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="B63" t="s">
-        <v>230</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -3173,90 +3150,90 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="2" max="2" width="26.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>168</v>
+        <v>221</v>
       </c>
       <c r="B1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>232</v>
+        <v>285</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>234</v>
+        <v>287</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>236</v>
+        <v>289</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>238</v>
+        <v>291</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>240</v>
+        <v>293</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>242</v>
+        <v>295</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>244</v>
+        <v>297</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>246</v>
+        <v>299</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>248</v>
+        <v>301</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>249</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -3270,62 +3247,62 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>250</v>
+        <v>303</v>
       </c>
       <c r="C1" t="s">
-        <v>251</v>
+        <v>304</v>
       </c>
       <c r="D1" t="s">
-        <v>252</v>
+        <v>305</v>
       </c>
       <c r="E1" t="s">
-        <v>253</v>
+        <v>306</v>
       </c>
       <c r="F1" t="s">
-        <v>254</v>
+        <v>307</v>
       </c>
       <c r="G1" t="s">
-        <v>255</v>
+        <v>308</v>
       </c>
       <c r="H1" t="s">
-        <v>256</v>
+        <v>309</v>
       </c>
       <c r="I1" t="s">
-        <v>257</v>
+        <v>310</v>
       </c>
       <c r="J1" t="s">
-        <v>258</v>
+        <v>311</v>
       </c>
       <c r="K1" t="s">
-        <v>259</v>
+        <v>312</v>
       </c>
       <c r="L1" t="s">
-        <v>260</v>
+        <v>313</v>
       </c>
       <c r="M1" t="s">
-        <v>261</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -3339,250 +3316,250 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>262</v>
+        <v>315</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>263</v>
+        <v>316</v>
       </c>
       <c r="B2" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>265</v>
+        <v>318</v>
       </c>
       <c r="B3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>267</v>
+        <v>320</v>
       </c>
       <c r="B4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>269</v>
+        <v>322</v>
       </c>
       <c r="B5" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>271</v>
+        <v>324</v>
       </c>
       <c r="B6" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>273</v>
+        <v>326</v>
       </c>
       <c r="B7" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>275</v>
+        <v>328</v>
       </c>
       <c r="B8" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>277</v>
+        <v>330</v>
       </c>
       <c r="B9" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>279</v>
+        <v>332</v>
       </c>
       <c r="B10" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>281</v>
+        <v>334</v>
       </c>
       <c r="B11" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>283</v>
+        <v>336</v>
       </c>
       <c r="B12" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>285</v>
+        <v>338</v>
       </c>
       <c r="B13" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>287</v>
+        <v>340</v>
       </c>
       <c r="B14" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>289</v>
+        <v>342</v>
       </c>
       <c r="B15" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>291</v>
+        <v>344</v>
       </c>
       <c r="B16" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>293</v>
+        <v>346</v>
       </c>
       <c r="B17" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>295</v>
+        <v>348</v>
       </c>
       <c r="B18" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>297</v>
+        <v>350</v>
       </c>
       <c r="B19" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>299</v>
+        <v>352</v>
       </c>
       <c r="B20" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>301</v>
+        <v>354</v>
       </c>
       <c r="B21" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>303</v>
+        <v>356</v>
       </c>
       <c r="B22" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>305</v>
+        <v>358</v>
       </c>
       <c r="B23" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>307</v>
+        <v>360</v>
       </c>
       <c r="B24" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>309</v>
+        <v>362</v>
       </c>
       <c r="B25" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>311</v>
+        <v>364</v>
       </c>
       <c r="B26" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>313</v>
+        <v>366</v>
       </c>
       <c r="B27" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>315</v>
+        <v>368</v>
       </c>
       <c r="B28" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>317</v>
+        <v>370</v>
       </c>
       <c r="B29" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>319</v>
+        <v>372</v>
       </c>
       <c r="B30" t="s">
-        <v>320</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
canvis en la forma d'afegir una correcció manual
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -39,12 +39,6 @@
       <name val="Aptos Narrow"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
@@ -104,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="center"/>
@@ -116,8 +110,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -593,76 +586,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>game_code</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>code_h</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>code_a</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>round</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>data_entry</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>caller_1</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>caller_2</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>timer</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>shot_clock_operator</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>irs_operator</t>
         </is>
       </c>
-      <c r="N1" s="8" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>is_processed</t>
         </is>
@@ -1091,7 +1084,7 @@
         </is>
       </c>
       <c r="N8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1229,6 +1222,64 @@
         </is>
       </c>
       <c r="N11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>U2025_170</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LKB</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>NIO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" t="n">
+        <v>17</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>DOVILE RUSONYTE</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>RASA KIZIKAITE</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>AUKSE ZAKRIENE</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ODETA DULIENE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>VIDAS MACYS</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
script per a inserir partits a través de la api oficial
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1339,6 +1339,4642 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>U2025_177</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NIO</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BES</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" t="n">
+        <v>18</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>U2025_171</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>WRO</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LJU</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" t="n">
+        <v>18</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>U2025_179</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TRN</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ULM</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" t="n">
+        <v>18</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>U2025_178</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TTK</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>NIN</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>11</v>
+      </c>
+      <c r="G16" t="n">
+        <v>18</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>U2025_174</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CLU</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ARI</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>11</v>
+      </c>
+      <c r="G17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>U2025_180</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BUD</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BOU</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>11</v>
+      </c>
+      <c r="G18" t="n">
+        <v>18</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>U2025_175</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>KLA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BAH</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="n">
+        <v>11</v>
+      </c>
+      <c r="G19" t="n">
+        <v>18</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>U2025_172</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HAM</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>11</v>
+      </c>
+      <c r="G20" t="n">
+        <v>18</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>U2025_173</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>VNC</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>JER</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>11</v>
+      </c>
+      <c r="G21" t="n">
+        <v>18</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>U2025_176</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LLI</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LKB</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>11</v>
+      </c>
+      <c r="G22" t="n">
+        <v>18</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E2025_271</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>12</v>
+      </c>
+      <c r="G23" t="n">
+        <v>28</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E2025_273</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12</v>
+      </c>
+      <c r="G24" t="n">
+        <v>28</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E2025_272</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>12</v>
+      </c>
+      <c r="G25" t="n">
+        <v>28</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E2025_275</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="n">
+        <v>12</v>
+      </c>
+      <c r="G26" t="n">
+        <v>28</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E2025_274</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>12</v>
+      </c>
+      <c r="G27" t="n">
+        <v>28</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E2025_280</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>13</v>
+      </c>
+      <c r="G28" t="n">
+        <v>28</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E2025_277</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>13</v>
+      </c>
+      <c r="G29" t="n">
+        <v>28</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E2025_279</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>13</v>
+      </c>
+      <c r="G30" t="n">
+        <v>28</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E2025_278</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>13</v>
+      </c>
+      <c r="G31" t="n">
+        <v>28</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>E2025_276</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G32" t="n">
+        <v>28</v>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>E2025_281</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>25</v>
+      </c>
+      <c r="G33" t="n">
+        <v>29</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>E2025_283</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>25</v>
+      </c>
+      <c r="G34" t="n">
+        <v>29</v>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>E2025_286</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="n">
+        <v>25</v>
+      </c>
+      <c r="G35" t="n">
+        <v>29</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>E2025_282</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>25</v>
+      </c>
+      <c r="G36" t="n">
+        <v>29</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>E2025_287</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>26</v>
+      </c>
+      <c r="G37" t="n">
+        <v>29</v>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>E2025_284</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="n">
+        <v>26</v>
+      </c>
+      <c r="G38" t="n">
+        <v>29</v>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>E2025_288</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>26</v>
+      </c>
+      <c r="G39" t="n">
+        <v>29</v>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>E2025_289</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>26</v>
+      </c>
+      <c r="G40" t="n">
+        <v>29</v>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>E2025_285</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>26</v>
+      </c>
+      <c r="G41" t="n">
+        <v>29</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>E2025_290</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>26</v>
+      </c>
+      <c r="G42" t="n">
+        <v>29</v>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>E2025_205</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" t="n">
+        <v>21</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>E2025_292</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" t="n">
+        <v>5</v>
+      </c>
+      <c r="G44" t="n">
+        <v>30</v>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>E2025_293</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>5</v>
+      </c>
+      <c r="G45" t="n">
+        <v>30</v>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>E2025_296</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>30</v>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>E2025_294</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" t="n">
+        <v>30</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>E2025_291</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>5</v>
+      </c>
+      <c r="G48" t="n">
+        <v>30</v>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>E2025_295</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5</v>
+      </c>
+      <c r="G49" t="n">
+        <v>30</v>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>E2025_297</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" t="n">
+        <v>6</v>
+      </c>
+      <c r="G50" t="n">
+        <v>30</v>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>E2025_299</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" t="n">
+        <v>6</v>
+      </c>
+      <c r="G51" t="n">
+        <v>30</v>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>E2025_300</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" t="n">
+        <v>30</v>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>E2025_298</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E53" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" t="n">
+        <v>6</v>
+      </c>
+      <c r="G53" t="n">
+        <v>30</v>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>E2025_334</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" t="n">
+        <v>10</v>
+      </c>
+      <c r="G54" t="n">
+        <v>34</v>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>E2025_308</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E55" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" t="n">
+        <v>12</v>
+      </c>
+      <c r="G55" t="n">
+        <v>31</v>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>E2025_306</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" t="n">
+        <v>12</v>
+      </c>
+      <c r="G56" t="n">
+        <v>31</v>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>E2025_305</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E57" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" t="n">
+        <v>12</v>
+      </c>
+      <c r="G57" t="n">
+        <v>31</v>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>E2025_304</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E58" t="n">
+        <v>3</v>
+      </c>
+      <c r="F58" t="n">
+        <v>12</v>
+      </c>
+      <c r="G58" t="n">
+        <v>31</v>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>E2025_301</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E59" t="n">
+        <v>3</v>
+      </c>
+      <c r="F59" t="n">
+        <v>12</v>
+      </c>
+      <c r="G59" t="n">
+        <v>31</v>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>E2025_303</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E60" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" t="n">
+        <v>12</v>
+      </c>
+      <c r="G60" t="n">
+        <v>31</v>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>E2025_302</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F61" t="n">
+        <v>12</v>
+      </c>
+      <c r="G61" t="n">
+        <v>31</v>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>E2025_307</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E62" t="n">
+        <v>3</v>
+      </c>
+      <c r="F62" t="n">
+        <v>13</v>
+      </c>
+      <c r="G62" t="n">
+        <v>31</v>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>E2025_310</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F63" t="n">
+        <v>13</v>
+      </c>
+      <c r="G63" t="n">
+        <v>31</v>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>E2025_309</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" t="n">
+        <v>13</v>
+      </c>
+      <c r="G64" t="n">
+        <v>31</v>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>E2025_134</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E65" t="n">
+        <v>3</v>
+      </c>
+      <c r="F65" t="n">
+        <v>17</v>
+      </c>
+      <c r="G65" t="n">
+        <v>14</v>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>E2025_316</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E66" t="n">
+        <v>3</v>
+      </c>
+      <c r="F66" t="n">
+        <v>19</v>
+      </c>
+      <c r="G66" t="n">
+        <v>32</v>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>E2025_312</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E67" t="n">
+        <v>3</v>
+      </c>
+      <c r="F67" t="n">
+        <v>19</v>
+      </c>
+      <c r="G67" t="n">
+        <v>32</v>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>E2025_313</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E68" t="n">
+        <v>3</v>
+      </c>
+      <c r="F68" t="n">
+        <v>19</v>
+      </c>
+      <c r="G68" t="n">
+        <v>32</v>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>E2025_315</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F69" t="n">
+        <v>19</v>
+      </c>
+      <c r="G69" t="n">
+        <v>32</v>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>E2025_311</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F70" t="n">
+        <v>19</v>
+      </c>
+      <c r="G70" t="n">
+        <v>32</v>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>E2025_314</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E71" t="n">
+        <v>3</v>
+      </c>
+      <c r="F71" t="n">
+        <v>19</v>
+      </c>
+      <c r="G71" t="n">
+        <v>32</v>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>E2025_317</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E72" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" t="n">
+        <v>20</v>
+      </c>
+      <c r="G72" t="n">
+        <v>32</v>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>E2025_320</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E73" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" t="n">
+        <v>20</v>
+      </c>
+      <c r="G73" t="n">
+        <v>32</v>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>E2025_318</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E74" t="n">
+        <v>3</v>
+      </c>
+      <c r="F74" t="n">
+        <v>20</v>
+      </c>
+      <c r="G74" t="n">
+        <v>32</v>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>E2025_319</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E75" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" t="n">
+        <v>20</v>
+      </c>
+      <c r="G75" t="n">
+        <v>32</v>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>E2025_322</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E76" t="n">
+        <v>3</v>
+      </c>
+      <c r="F76" t="n">
+        <v>24</v>
+      </c>
+      <c r="G76" t="n">
+        <v>33</v>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>E2025_329</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" t="n">
+        <v>24</v>
+      </c>
+      <c r="G77" t="n">
+        <v>33</v>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>E2025_324</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E78" t="n">
+        <v>3</v>
+      </c>
+      <c r="F78" t="n">
+        <v>24</v>
+      </c>
+      <c r="G78" t="n">
+        <v>33</v>
+      </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>E2025_321</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E79" t="n">
+        <v>3</v>
+      </c>
+      <c r="F79" t="n">
+        <v>24</v>
+      </c>
+      <c r="G79" t="n">
+        <v>33</v>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>E2025_327</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E80" t="n">
+        <v>3</v>
+      </c>
+      <c r="F80" t="n">
+        <v>24</v>
+      </c>
+      <c r="G80" t="n">
+        <v>33</v>
+      </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
+      <c r="N80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>E2025_325</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F81" t="n">
+        <v>24</v>
+      </c>
+      <c r="G81" t="n">
+        <v>33</v>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>E2025_323</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E82" t="n">
+        <v>3</v>
+      </c>
+      <c r="F82" t="n">
+        <v>24</v>
+      </c>
+      <c r="G82" t="n">
+        <v>33</v>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
+      <c r="N82" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>E2025_326</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E83" t="n">
+        <v>3</v>
+      </c>
+      <c r="F83" t="n">
+        <v>24</v>
+      </c>
+      <c r="G83" t="n">
+        <v>33</v>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
+      <c r="N83" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>E2025_330</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E84" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" t="n">
+        <v>25</v>
+      </c>
+      <c r="G84" t="n">
+        <v>33</v>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>E2025_333</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E85" t="n">
+        <v>3</v>
+      </c>
+      <c r="F85" t="n">
+        <v>26</v>
+      </c>
+      <c r="G85" t="n">
+        <v>34</v>
+      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
+      <c r="N85" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>E2025_332</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E86" t="n">
+        <v>3</v>
+      </c>
+      <c r="F86" t="n">
+        <v>26</v>
+      </c>
+      <c r="G86" t="n">
+        <v>34</v>
+      </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
+      <c r="N86" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>E2025_331</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E87" t="n">
+        <v>3</v>
+      </c>
+      <c r="F87" t="n">
+        <v>26</v>
+      </c>
+      <c r="G87" t="n">
+        <v>34</v>
+      </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
+      <c r="N87" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>E2025_335</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E88" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" t="n">
+        <v>26</v>
+      </c>
+      <c r="G88" t="n">
+        <v>34</v>
+      </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
+      <c r="N88" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>E2025_338</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E89" t="n">
+        <v>3</v>
+      </c>
+      <c r="F89" t="n">
+        <v>27</v>
+      </c>
+      <c r="G89" t="n">
+        <v>34</v>
+      </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
+      <c r="N89" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>E2025_339</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E90" t="n">
+        <v>3</v>
+      </c>
+      <c r="F90" t="n">
+        <v>27</v>
+      </c>
+      <c r="G90" t="n">
+        <v>34</v>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
+      <c r="N90" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>E2025_340</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E91" t="n">
+        <v>3</v>
+      </c>
+      <c r="F91" t="n">
+        <v>27</v>
+      </c>
+      <c r="G91" t="n">
+        <v>34</v>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
+      <c r="N91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>E2025_337</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F92" t="n">
+        <v>27</v>
+      </c>
+      <c r="G92" t="n">
+        <v>34</v>
+      </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
+      <c r="N92" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>E2025_336</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E93" t="n">
+        <v>3</v>
+      </c>
+      <c r="F93" t="n">
+        <v>27</v>
+      </c>
+      <c r="G93" t="n">
+        <v>34</v>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
+      <c r="N93" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>E2025_328</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E94" t="n">
+        <v>3</v>
+      </c>
+      <c r="F94" t="n">
+        <v>31</v>
+      </c>
+      <c r="G94" t="n">
+        <v>33</v>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>E2025_348</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E95" t="n">
+        <v>4</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" t="n">
+        <v>35</v>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>E2025_341</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E96" t="n">
+        <v>4</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" t="n">
+        <v>35</v>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>E2025_345</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E97" t="n">
+        <v>4</v>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
+      </c>
+      <c r="G97" t="n">
+        <v>35</v>
+      </c>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>E2025_342</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E98" t="n">
+        <v>4</v>
+      </c>
+      <c r="F98" t="n">
+        <v>2</v>
+      </c>
+      <c r="G98" t="n">
+        <v>35</v>
+      </c>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>E2025_343</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E99" t="n">
+        <v>4</v>
+      </c>
+      <c r="F99" t="n">
+        <v>2</v>
+      </c>
+      <c r="G99" t="n">
+        <v>35</v>
+      </c>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>E2025_344</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E100" t="n">
+        <v>4</v>
+      </c>
+      <c r="F100" t="n">
+        <v>2</v>
+      </c>
+      <c r="G100" t="n">
+        <v>35</v>
+      </c>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>E2025_347</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E101" t="n">
+        <v>4</v>
+      </c>
+      <c r="F101" t="n">
+        <v>3</v>
+      </c>
+      <c r="G101" t="n">
+        <v>35</v>
+      </c>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>E2025_349</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E102" t="n">
+        <v>4</v>
+      </c>
+      <c r="F102" t="n">
+        <v>3</v>
+      </c>
+      <c r="G102" t="n">
+        <v>35</v>
+      </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>E2025_350</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F103" t="n">
+        <v>3</v>
+      </c>
+      <c r="G103" t="n">
+        <v>35</v>
+      </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>E2025_346</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E104" t="n">
+        <v>4</v>
+      </c>
+      <c r="F104" t="n">
+        <v>3</v>
+      </c>
+      <c r="G104" t="n">
+        <v>35</v>
+      </c>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
+      <c r="N104" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>E2025_354</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E105" t="n">
+        <v>4</v>
+      </c>
+      <c r="F105" t="n">
+        <v>7</v>
+      </c>
+      <c r="G105" t="n">
+        <v>36</v>
+      </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
+      <c r="N105" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>E2025_358</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E106" t="n">
+        <v>4</v>
+      </c>
+      <c r="F106" t="n">
+        <v>7</v>
+      </c>
+      <c r="G106" t="n">
+        <v>36</v>
+      </c>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
+      <c r="N106" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>E2025_352</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E107" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" t="n">
+        <v>7</v>
+      </c>
+      <c r="G107" t="n">
+        <v>36</v>
+      </c>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>E2025_355</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E108" t="n">
+        <v>4</v>
+      </c>
+      <c r="F108" t="n">
+        <v>7</v>
+      </c>
+      <c r="G108" t="n">
+        <v>36</v>
+      </c>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
+      <c r="N108" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>E2025_357</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E109" t="n">
+        <v>4</v>
+      </c>
+      <c r="F109" t="n">
+        <v>7</v>
+      </c>
+      <c r="G109" t="n">
+        <v>36</v>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
+      <c r="N109" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>E2025_356</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E110" t="n">
+        <v>4</v>
+      </c>
+      <c r="F110" t="n">
+        <v>7</v>
+      </c>
+      <c r="G110" t="n">
+        <v>36</v>
+      </c>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
+      <c r="N110" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>E2025_353</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E111" t="n">
+        <v>4</v>
+      </c>
+      <c r="F111" t="n">
+        <v>7</v>
+      </c>
+      <c r="G111" t="n">
+        <v>36</v>
+      </c>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>E2025_351</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E112" t="n">
+        <v>4</v>
+      </c>
+      <c r="F112" t="n">
+        <v>7</v>
+      </c>
+      <c r="G112" t="n">
+        <v>36</v>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
+      <c r="N112" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>E2025_360</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E113" t="n">
+        <v>4</v>
+      </c>
+      <c r="F113" t="n">
+        <v>8</v>
+      </c>
+      <c r="G113" t="n">
+        <v>36</v>
+      </c>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>E2025_359</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E114" t="n">
+        <v>4</v>
+      </c>
+      <c r="F114" t="n">
+        <v>8</v>
+      </c>
+      <c r="G114" t="n">
+        <v>36</v>
+      </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>E2025_362</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E115" t="n">
+        <v>4</v>
+      </c>
+      <c r="F115" t="n">
+        <v>9</v>
+      </c>
+      <c r="G115" t="n">
+        <v>37</v>
+      </c>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>E2025_363</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E116" t="n">
+        <v>4</v>
+      </c>
+      <c r="F116" t="n">
+        <v>9</v>
+      </c>
+      <c r="G116" t="n">
+        <v>37</v>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
+      <c r="N116" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>E2025_361</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E117" t="n">
+        <v>4</v>
+      </c>
+      <c r="F117" t="n">
+        <v>9</v>
+      </c>
+      <c r="G117" t="n">
+        <v>37</v>
+      </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
+      <c r="N117" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>E2025_365</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E118" t="n">
+        <v>4</v>
+      </c>
+      <c r="F118" t="n">
+        <v>9</v>
+      </c>
+      <c r="G118" t="n">
+        <v>37</v>
+      </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
+      <c r="N118" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>E2025_364</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E119" t="n">
+        <v>4</v>
+      </c>
+      <c r="F119" t="n">
+        <v>9</v>
+      </c>
+      <c r="G119" t="n">
+        <v>37</v>
+      </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
+      <c r="N119" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>E2025_367</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E120" t="n">
+        <v>4</v>
+      </c>
+      <c r="F120" t="n">
+        <v>10</v>
+      </c>
+      <c r="G120" t="n">
+        <v>37</v>
+      </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
+      <c r="N120" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>E2025_366</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E121" t="n">
+        <v>4</v>
+      </c>
+      <c r="F121" t="n">
+        <v>10</v>
+      </c>
+      <c r="G121" t="n">
+        <v>37</v>
+      </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
+      <c r="N121" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>E2025_368</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E122" t="n">
+        <v>4</v>
+      </c>
+      <c r="F122" t="n">
+        <v>10</v>
+      </c>
+      <c r="G122" t="n">
+        <v>37</v>
+      </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
+      <c r="N122" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>E2025_370</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E123" t="n">
+        <v>4</v>
+      </c>
+      <c r="F123" t="n">
+        <v>10</v>
+      </c>
+      <c r="G123" t="n">
+        <v>37</v>
+      </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
+      <c r="N123" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>E2025_369</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E124" t="n">
+        <v>4</v>
+      </c>
+      <c r="F124" t="n">
+        <v>10</v>
+      </c>
+      <c r="G124" t="n">
+        <v>37</v>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
+      <c r="N124" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>E2025_371</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>ASV</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>ULK</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E125" t="n">
+        <v>4</v>
+      </c>
+      <c r="F125" t="n">
+        <v>16</v>
+      </c>
+      <c r="G125" t="n">
+        <v>38</v>
+      </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>E2025_372</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>TEL</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>VIR</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E126" t="n">
+        <v>4</v>
+      </c>
+      <c r="F126" t="n">
+        <v>16</v>
+      </c>
+      <c r="G126" t="n">
+        <v>38</v>
+      </c>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
+      <c r="N126" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>E2025_375</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>OLY</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E127" t="n">
+        <v>4</v>
+      </c>
+      <c r="F127" t="n">
+        <v>16</v>
+      </c>
+      <c r="G127" t="n">
+        <v>38</v>
+      </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>E2025_373</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>BAS</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E128" t="n">
+        <v>4</v>
+      </c>
+      <c r="F128" t="n">
+        <v>16</v>
+      </c>
+      <c r="G128" t="n">
+        <v>38</v>
+      </c>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>E2025_374</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>MAD</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E129" t="n">
+        <v>4</v>
+      </c>
+      <c r="F129" t="n">
+        <v>16</v>
+      </c>
+      <c r="G129" t="n">
+        <v>38</v>
+      </c>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
+      <c r="N129" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>E2025_378</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>PAM</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E130" t="n">
+        <v>4</v>
+      </c>
+      <c r="F130" t="n">
+        <v>17</v>
+      </c>
+      <c r="G130" t="n">
+        <v>38</v>
+      </c>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
+      <c r="N130" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>E2025_380</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ZAL</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>PRS</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E131" t="n">
+        <v>4</v>
+      </c>
+      <c r="F131" t="n">
+        <v>17</v>
+      </c>
+      <c r="G131" t="n">
+        <v>38</v>
+      </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
+      <c r="N131" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>E2025_377</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>HTA</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E132" t="n">
+        <v>4</v>
+      </c>
+      <c r="F132" t="n">
+        <v>17</v>
+      </c>
+      <c r="G132" t="n">
+        <v>38</v>
+      </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
+      <c r="N132" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>E2025_376</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>IST</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E133" t="n">
+        <v>4</v>
+      </c>
+      <c r="F133" t="n">
+        <v>17</v>
+      </c>
+      <c r="G133" t="n">
+        <v>38</v>
+      </c>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
+      <c r="N133" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>E2025_379</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>MUN</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E134" t="n">
+        <v>4</v>
+      </c>
+      <c r="F134" t="n">
+        <v>17</v>
+      </c>
+      <c r="G134" t="n">
+        <v>38</v>
+      </c>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
+      <c r="N134" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
canvis en processament de correccions i principi arxiu per extreure dades de uscs de la api
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -37,20 +37,8 @@
     </font>
     <font>
       <name val="Aptos Narrow"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
@@ -110,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="justify" vertical="center"/>
@@ -119,12 +107,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -604,72 +590,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>game_code</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>code_h</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>code_a</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>round</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>data_entry</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>caller_1</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>caller_2</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>timer</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>shot_clock_operator</t>
         </is>
       </c>
-      <c r="M1" s="9" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>irs_operator</t>
         </is>
       </c>
-      <c r="N1" s="9" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>is_processed</t>
         </is>
@@ -1376,7 +1362,7 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1407,14 +1393,34 @@
       <c r="G14" t="n">
         <v>18</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>AGNIESZKA WYSOCKA</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>DOROTA RECZUCH</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>KATARZYNA LESIECKA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ALEKSANDRA LASKOWSKA</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>MATEUSZ KOJKA</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -5989,14 +5995,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I41"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="12.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="27.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="14.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="20.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="12.1640625" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="45.1640625" customWidth="1" min="9" max="9"/>
+    <col width="12.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="27.6328125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="14.1796875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="20.36328125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12.1796875" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="45.1796875" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6917,10 +6923,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="34.6640625" customWidth="1" min="2" max="2"/>
+    <col width="34.6328125" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7694,10 +7700,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="16.5" customWidth="1" min="1" max="1"/>
-    <col width="26.33203125" customWidth="1" min="2" max="2"/>
+    <col width="16.453125" customWidth="1" min="1" max="1"/>
+    <col width="26.36328125" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7835,21 +7841,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="12.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="7.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="9.5" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="10.1640625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="12.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.36328125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.36328125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.453125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.36328125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.1796875" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="12.6328125" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="7" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="7.6640625" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="8.6640625" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="10.33203125" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="13.83203125" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="11.83203125" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="18.83203125" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="7.6328125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="8.6328125" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="10.36328125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13.81640625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="11.81640625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="18.81640625" bestFit="1" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7934,10 +7940,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="10.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="13.5" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="17.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="13.453125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.6328125" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
agafar uscs de temporada del endpoint season people
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" state="visible" r:id="rId1"/>
@@ -211,11 +211,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table3" displayName="Table3" ref="A1:B63" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:B63"/>
-  <tableColumns count="2">
-    <tableColumn id="1" name="team_code"/>
-    <tableColumn id="2" name="name"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table3" displayName="Table3" ref="A1:C63" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:C63"/>
+  <tableColumns count="3">
+    <tableColumn id="3" name="code"/>
+    <tableColumn id="1" name="name"/>
+    <tableColumn id="2" name="team_code"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5995,14 +5996,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I41"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="12.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="27.6328125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="14.1796875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="20.36328125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="12.1796875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="45.1796875" customWidth="1" min="9" max="9"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="27.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="14.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="20.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="45.1640625" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6922,768 +6923,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C54"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="34.6328125" customWidth="1" min="2" max="2"/>
+    <col width="7.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="8" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="34.6640625" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>team_code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>DYLAN YAMDJEU SANGOUNGOU</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>JIMMY MOLLET</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>BASTIEN BONNETON</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>CYRIL LONGELIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>MAGALI CARTIER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>AXEL QUENEY</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>BRIAN PETER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DJAMEL SOUDANI</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CHRISTIAN MOLLET</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>SANDRA PRINCELLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>PATRICK JOLIVET</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>PRS</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PIERRE BERNARDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>JESUS LOPEZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>POL FRANQUESA</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>ROBERTO BAÑOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>MARC BAYO</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>LLUIS ESPINOSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>RICARD MONGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>MARIA JOSE SERRANO</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>CARLOS MARTIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>MANEL LUENGO</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>FRANCIS RUIZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>ADRIA RUBIROLA</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>LAILA GONELL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>NEŽA JUG</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>ZIGA JANEZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>ALENKA MARKIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>SILVO MARKIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>KARMEN BELSAK</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>MATJAZ PODLESNIK</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>GORAN HODZIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>ANA JUG</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>MATIC MARKIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>ANDREJ STRUKELJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>URBAN VERBIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>GASPER KOLMAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>LJU</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>ZIGA BENKO</t>
-        </is>
-      </c>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B39" s="1" t="inlineStr">
-        <is>
-          <t>MILOS MOSIC</t>
-        </is>
-      </c>
+      <c r="C39" s="1" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B40" s="1" t="inlineStr">
-        <is>
-          <t>IVAN MOSIC</t>
-        </is>
-      </c>
+      <c r="C40" s="1" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B41" s="1" t="inlineStr">
-        <is>
-          <t>MIODRAG STOJANOVIC</t>
-        </is>
-      </c>
+      <c r="C41" s="1" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>PETAR VASILJEVIC</t>
-        </is>
-      </c>
+      <c r="C42" s="1" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>PREDRAG VASILJEVIC</t>
-        </is>
-      </c>
+      <c r="C43" s="1" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B44" s="1" t="inlineStr">
-        <is>
-          <t>IVANA VASILJEVIC</t>
-        </is>
-      </c>
+      <c r="C44" s="1" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B45" s="1" t="inlineStr">
-        <is>
-          <t>MILICA STOSIC</t>
-        </is>
-      </c>
+      <c r="C45" s="1" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B46" s="1" t="inlineStr">
-        <is>
-          <t>JOVANA VESKOVIC</t>
-        </is>
-      </c>
+      <c r="C46" s="1" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B47" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ANA KRSTIC </t>
-        </is>
-      </c>
+      <c r="C47" s="1" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>MILAN KVRGIC</t>
-        </is>
-      </c>
+      <c r="C48" s="1" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B49" s="1" t="inlineStr">
-        <is>
-          <t>LUKA ANDRIC</t>
-        </is>
-      </c>
+      <c r="C49" s="1" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B50" s="1" t="inlineStr">
-        <is>
-          <t>MARKO BOZIC</t>
-        </is>
-      </c>
+      <c r="C50" s="1" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t>SARA PROJOVIC</t>
-        </is>
-      </c>
+      <c r="C51" s="1" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>MARIJA SAVIC</t>
-        </is>
-      </c>
+      <c r="C52" s="1" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>JER</t>
-        </is>
-      </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>SARA MILICIC</t>
-        </is>
-      </c>
+      <c r="C53" s="1" t="n"/>
     </row>
     <row r="54" ht="16" customHeight="1">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t>ELOI V</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>ELOI VV</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>ELOI VVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>ELOI VVVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>ELOI VVVVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>ELOI VVVVVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>ELOI VVVVVVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>ELOI VVVVVVVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>ELOI VVVVVVVVV</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>TTK</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>ELOI VVVVVVVVVV</t>
-        </is>
-      </c>
+      <c r="C54" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7700,10 +7012,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="16.453125" customWidth="1" min="1" max="1"/>
-    <col width="26.36328125" customWidth="1" min="2" max="2"/>
+    <col width="16.5" customWidth="1" min="1" max="1"/>
+    <col width="26.33203125" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7841,21 +7153,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="12.36328125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="7.36328125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="9.453125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.36328125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="10.1796875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="12.6328125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="12.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="7" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="7.6328125" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="8.6328125" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="10.36328125" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="13.81640625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="11.81640625" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="18.81640625" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="18.83203125" bestFit="1" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7940,10 +7252,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="13.453125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="17.6328125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
dades correccions partits divendres 13 de febrer
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N134"/>
+  <dimension ref="A1:N138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2029,7 +2029,7 @@
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2067,7 +2067,7 @@
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2105,7 +2105,7 @@
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -5981,6 +5981,158 @@
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr"/>
       <c r="N134" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>U2025_182</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>TTK</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E135" t="n">
+        <v>3</v>
+      </c>
+      <c r="F135" t="n">
+        <v>11</v>
+      </c>
+      <c r="G135" t="n">
+        <v>19</v>
+      </c>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
+      <c r="N135" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>U2025_183</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>BUD</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CLU</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E136" t="n">
+        <v>3</v>
+      </c>
+      <c r="F136" t="n">
+        <v>11</v>
+      </c>
+      <c r="G136" t="n">
+        <v>19</v>
+      </c>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr"/>
+      <c r="N136" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>U2025_181</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>LJU</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>NIN</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E137" t="n">
+        <v>3</v>
+      </c>
+      <c r="F137" t="n">
+        <v>11</v>
+      </c>
+      <c r="G137" t="n">
+        <v>19</v>
+      </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
+      <c r="M137" t="inlineStr"/>
+      <c r="N137" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>U2025_184</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>VNC</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>TRN</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E138" t="n">
+        <v>3</v>
+      </c>
+      <c r="F138" t="n">
+        <v>11</v>
+      </c>
+      <c r="G138" t="n">
+        <v>19</v>
+      </c>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr"/>
+      <c r="N138" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new games from round 29 (day 25, february)
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" state="visible" r:id="rId1"/>
@@ -2143,7 +2143,7 @@
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2181,7 +2181,7 @@
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -2219,7 +2219,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>1438645665340198915</t>
+          <t>884934005005373460</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
corrections from 3 games on february 26 plus fixing the excel_to_db file to ignore usc table
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -2333,7 +2333,7 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2447,7 +2447,7 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
afegit botó per a que cada usuari pugui processar les correccions des dels seus dispositius
</commit_message>
<xml_diff>
--- a/reports_automation_database.xlsx
+++ b/reports_automation_database.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Game" sheetId="1" state="visible" r:id="rId1"/>
@@ -2371,7 +2371,7 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -6148,14 +6148,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I41"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="12.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="27.6328125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="14.1796875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="20.36328125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="12.1796875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="45.1796875" customWidth="1" min="9" max="9"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="27.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="14.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="20.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="45.1640625" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7076,12 +7076,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C54"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="7.453125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.5" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="8" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="12.1796875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="34.6328125" customWidth="1" min="4" max="4"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="34.6640625" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7164,10 +7164,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="16.453125" customWidth="1" min="1" max="1"/>
-    <col width="26.36328125" customWidth="1" min="2" max="2"/>
+    <col width="16.5" customWidth="1" min="1" max="1"/>
+    <col width="26.33203125" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7305,21 +7305,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="12.36328125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="7.36328125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="9.453125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.36328125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="10.1796875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="12.6328125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.33203125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="12.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="7" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="7.6328125" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="8.6328125" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="10.36328125" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="13.81640625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="11.81640625" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="18.81640625" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="8.6640625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13.83203125" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="18.83203125" bestFit="1" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7404,10 +7404,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="13.453125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="17.6328125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.6640625" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>